<commit_message>
Panoplies : rebalance bonus + rename Acier → Fer
Sur retour utilisateur, ajustements des bonus de panoplie :

- 🛡️ Acier → Fer (renommage, code 'iron' inchangé) — bonus défense
  conservés : +1 / +2 / +5 / +8

- 🟫 Cuir : passe de "esquive" à "PV max"
  → +4 / +8 / +20 / +32 PV
  Plus thématique (le cuir protège, ne fait pas esquiver)

- 🟢 Slime : régénération PV/min inchangée (+1 / +2 / +5 / +8)

- 👹 Gobeline : passe de "chance critique" à "dégâts critiques"
  → +1 / +2 / +4 / +8 % crit damage
  (frappe rare mais brutale, plutôt que crit fréquent)

- 🧵 Lin : passe de "dégâts critiques" à "esquive"
  → +1 / +2 / +3 / +5 % esquive
  (le tissu léger favorise l'agilité)

Tuto.txt + spreadsheet à jour. Tests : 344 passent.
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 2026-05-07 06:13 UTC</t>
+          <t>Généré le 2026-05-07 07:46 UTC</t>
         </is>
       </c>
     </row>
@@ -7859,7 +7859,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Acier</t>
+          <t>Fer</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -7917,27 +7917,27 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Souple et discret — favorise l'esquive.</t>
+          <t>Souple et résistant, renforce la vitalité du porteur.</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>dodge_flat +1</t>
+          <t>max_hp_flat +4</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>dodge_flat +2</t>
+          <t>max_hp_flat +8</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>dodge_flat +5</t>
+          <t>max_hp_flat +20</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>dodge_flat +8</t>
+          <t>max_hp_flat +32</t>
         </is>
       </c>
     </row>
@@ -8007,27 +8007,27 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Affutée par les fourbes habitudes des gobelins.</t>
+          <t>Affutée par les fourbes habitudes des gobelins — frappe rare mais brutale.</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>crit_chance_flat +1</t>
+          <t>crit_damage_flat +1</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>crit_chance_flat +2</t>
+          <t>crit_damage_flat +2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>crit_chance_flat +5</t>
+          <t>crit_damage_flat +4</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>crit_chance_flat +8</t>
+          <t>crit_damage_flat +8</t>
         </is>
       </c>
     </row>
@@ -8052,27 +8052,27 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>Tissu léger imprégné d'aura magique.</t>
+          <t>Tissu léger qui favorise l'agilité et l'esquive.</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>crit_damage_flat +1</t>
+          <t>dodge_flat +1</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>crit_damage_flat +2</t>
+          <t>dodge_flat +2</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>crit_damage_flat +5</t>
+          <t>dodge_flat +3</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>crit_damage_flat +8</t>
+          <t>dodge_flat +5</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Regen sakura_content.xlsx (19 nouveaux items + recettes panoplies)
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 2026-05-07 07:46 UTC</t>
+          <t>Généré le 2026-05-07 18:18 UTC</t>
         </is>
       </c>
     </row>
@@ -3398,12 +3398,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="23" customWidth="1" min="3" max="3"/>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="19" customWidth="1" min="6" max="6"/>
@@ -4636,6 +4636,1946 @@
           <t>slime_gel ×4
 wood_log ×3
 leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>gobelin_plastron_recipe</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Plastron gobelin</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>gobelin_plastron</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>chest</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>plastron</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×5
+iron_ingot ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_jambieres_recipe</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Jambières gobelin</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_jambieres</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>legs</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>jambieres</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×4
+iron_ingot ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>gobelin_bottes_recipe</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Bottes gobelin</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>gobelin_bottes</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>boots</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>bottes</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×3
+iron_ingot ×1
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_main_gauche_recipe</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Bouclier gobelin</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_main_gauche</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>main_gauche</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×3
+iron_ingot ×1
+wood_log ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>gobelin_bracelet_recipe</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Bracelet gobelin</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>gobelin_bracelet</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>bracelet</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>bracelet</t>
+        </is>
+      </c>
+      <c r="F39" t="n">
+        <v>1</v>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×2
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_ceinture_recipe</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Ceinture gobelin</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_ceinture</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>belt</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>ceinture</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×2
+iron_ingot ×1
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>gobelin_cape_recipe</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Cape gobelin</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>gobelin_cape</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>cape</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>cape</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×4
+linen_cloth ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_boucle_oreille_recipe</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Boucle gobelin</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_boucle_oreille</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>earring</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>boucle_oreille</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>iron_collier_recipe</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Collier en fer</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>iron_collier</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>necklace</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>collier</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>iron_ingot ×4
+polished_stone ×1
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>iron_ceinture_recipe</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Ceinture en fer</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>iron_ceinture</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>belt</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>ceinture</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
+          <t>iron_ingot ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>iron_cape_recipe</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Cape en fer</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>iron_cape</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>cape</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>cape</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>iron_ingot ×4
+linen_cloth ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>iron_boucle_oreille_recipe</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Boucle en fer</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>iron_boucle_oreille</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>earring</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>boucle_oreille</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
+          <t>iron_ingot ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>leather_main_droite_recipe</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Lame en cuir</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>leather_main_droite</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
+        <is>
+          <t>leather_strip ×3
+wood_log ×2
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
+          <t>leather_main_gauche_recipe</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Bouclier en cuir</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>leather_main_gauche</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>main_gauche</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
+          <t>leather_strip ×3
+wood_log ×3
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>leather_collier_recipe</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Collier en cuir</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>leather_collier</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>necklace</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>collier</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>leather_strip ×4
+polished_stone ×1
+linen_cloth ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="3" t="inlineStr">
+        <is>
+          <t>leather_bague_recipe</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Bague en cuir</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>leather_bague</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>ring</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>bague</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>leather_strip ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>leather_cape_recipe</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Cape en cuir</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>leather_cape</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>cape</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>cape</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
+        <is>
+          <t>leather_strip ×5
+linen_cloth ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="3" t="inlineStr">
+        <is>
+          <t>leather_boucle_oreille_recipe</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Boucle en cuir</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>leather_boucle_oreille</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>earring</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>boucle_oreille</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
+          <t>leather_strip ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>linen_jambieres_recipe</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>Jambières en lin</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>linen_jambieres</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>legs</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>jambieres</t>
+        </is>
+      </c>
+      <c r="F53" t="n">
+        <v>1</v>
+      </c>
+      <c r="G53" s="5" t="inlineStr">
+        <is>
+          <t>linen_cloth ×4
+leather_strip ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
+        <is>
+          <t>linen_bottes_recipe</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Bottes en lin</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>linen_bottes</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>boots</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>bottes</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
+          <t>linen_cloth ×3
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>linen_main_droite_recipe</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>Lame en lin</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>linen_main_droite</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
+        <is>
+          <t>linen_cloth ×3
+wood_log ×2
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
+        <is>
+          <t>linen_main_gauche_recipe</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Bouclier en lin</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>linen_main_gauche</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>main_gauche</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
+          <t>linen_cloth ×3
+wood_log ×3
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>linen_collier_recipe</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Collier en lin</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>linen_collier</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>necklace</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>collier</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>linen_cloth ×4
+polished_stone ×1
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
+        <is>
+          <t>linen_bague_recipe</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Bague en lin</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>linen_bague</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>ring</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>bague</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>linen_cloth ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>linen_ceinture_recipe</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Ceinture en lin</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>linen_ceinture</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>belt</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>ceinture</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
+        <is>
+          <t>linen_cloth ×2
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="3" t="inlineStr">
+        <is>
+          <t>linen_boucle_oreille_recipe</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Boucle en lin</t>
+        </is>
+      </c>
+      <c r="C60" s="3" t="inlineStr">
+        <is>
+          <t>linen_boucle_oreille</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>earring</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>boucle_oreille</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
+          <t>linen_cloth ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>slime_casque_recipe</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>Casque de slime</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>slime_casque</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>helmet</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>casque</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="5" t="inlineStr">
+        <is>
+          <t>slime_gel ×4
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="3" t="inlineStr">
+        <is>
+          <t>slime_plastron_recipe</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Plastron de slime</t>
+        </is>
+      </c>
+      <c r="C62" s="3" t="inlineStr">
+        <is>
+          <t>slime_plastron</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>chest</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>plastron</t>
+        </is>
+      </c>
+      <c r="F62" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
+          <t>slime_gel ×5
+leather_strip ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>slime_jambieres_recipe</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Jambières de slime</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>slime_jambieres</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>legs</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>jambieres</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>1</v>
+      </c>
+      <c r="G63" s="5" t="inlineStr">
+        <is>
+          <t>slime_gel ×4
+leather_strip ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="3" t="inlineStr">
+        <is>
+          <t>slime_bottes_recipe</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Bottes de slime</t>
+        </is>
+      </c>
+      <c r="C64" s="3" t="inlineStr">
+        <is>
+          <t>slime_bottes</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>boots</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>bottes</t>
+        </is>
+      </c>
+      <c r="F64" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
+          <t>slime_gel ×3
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>slime_bracelet_recipe</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Bracelet de slime</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>slime_bracelet</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>bracelet</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>bracelet</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>1</v>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>slime_gel ×2
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="3" t="inlineStr">
+        <is>
+          <t>slime_bague_recipe</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Bague de slime</t>
+        </is>
+      </c>
+      <c r="C66" s="3" t="inlineStr">
+        <is>
+          <t>slime_bague</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>ring</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>bague</t>
+        </is>
+      </c>
+      <c r="F66" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>slime_gel ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>slime_ceinture_recipe</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Ceinture de slime</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>slime_ceinture</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>belt</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ceinture</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>slime_gel ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="3" t="inlineStr">
+        <is>
+          <t>slime_boucle_oreille_recipe</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Boucle de slime</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>slime_boucle_oreille</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>earring</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>boucle_oreille</t>
+        </is>
+      </c>
+      <c r="F68" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
+          <t>slime_gel ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>iron_sword_recipe</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Épée en fer</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>iron_sword</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>iron_ingot ×3
+wood_log ×1
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>iron_warshield_recipe</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Pavois en fer</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>iron_warshield</t>
+        </is>
+      </c>
+      <c r="D70" s="3" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F70" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
+          <t>iron_ingot ×4
+leather_strip ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>iron_greatsword_recipe</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Espadon en fer</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>iron_greatsword</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>iron_ingot ×6
+wood_log ×3
+leather_strip ×3</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="3" t="inlineStr">
+        <is>
+          <t>iron_tower_shield_recipe</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Tour en fer</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>iron_tower_shield</t>
+        </is>
+      </c>
+      <c r="D72" s="3" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F72" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
+          <t>iron_ingot ×9
+leather_strip ×3</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>slime_morningstar_recipe</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Morningstar visqueuse</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>slime_morningstar</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>1</v>
+      </c>
+      <c r="G73" s="5" t="inlineStr">
+        <is>
+          <t>slime_gel ×3
+wood_log ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>slime_buckler_recipe</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Bouclier de gel</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>slime_buckler</t>
+        </is>
+      </c>
+      <c r="D74" s="3" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F74" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
+          <t>slime_gel ×3
+wood_log ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>slime_greatblade_recipe</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Lame visqueuse colossale</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>slime_greatblade</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>slime_gel ×9
+wood_log ×6
+iron_ingot ×3</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
+        <is>
+          <t>slime_tower_shield_recipe</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Tour de gel</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>slime_tower_shield</t>
+        </is>
+      </c>
+      <c r="D76" s="3" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F76" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
+          <t>slime_gel ×12
+wood_log ×9
+leather_strip ×3</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>gobelin_buckler_recipe</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Rondache gobeline</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>gobelin_buckler</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×3
+iron_ingot ×1
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_greataxe_recipe</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Grande hache gobeline</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_greataxe</t>
+        </is>
+      </c>
+      <c r="D78" s="3" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F78" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×12
+iron_ingot ×6
+wood_log ×3</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>gobelin_warshield_recipe</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Pavois gobelin</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>gobelin_warshield</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×9
+iron_ingot ×3
+wood_log ×6
+leather_strip ×3</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
+        <is>
+          <t>leather_dagger_recipe</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Dague en cuir</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>leather_dagger</t>
+        </is>
+      </c>
+      <c r="D80" s="3" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F80" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
+          <t>leather_strip ×2
+wood_log ×2
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>leather_buckler_recipe</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Rondache en cuir</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>leather_buckler</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
+        <is>
+          <t>leather_strip ×2
+wood_log ×2
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>leather_greatsword_recipe</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Grande lame en cuir</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>leather_greatsword</t>
+        </is>
+      </c>
+      <c r="D82" s="3" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F82" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
+          <t>leather_strip ×9
+wood_log ×6
+iron_ingot ×3</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>leather_tower_shield_recipe</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Tour en cuir</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>leather_tower_shield</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
+        <is>
+          <t>leather_strip ×9
+wood_log ×9
+iron_ingot ×3</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
+          <t>linen_rapier_recipe</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Rapière en lin</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>linen_rapier</t>
+        </is>
+      </c>
+      <c r="D84" s="3" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F84" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
+          <t>linen_cloth ×2
+wood_log ×2
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>linen_aegis_recipe</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Égide en lin</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>linen_aegis</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
+        <is>
+          <t>linen_cloth ×2
+wood_log ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
+        <is>
+          <t>linen_greatblade_recipe</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Grande lame en lin</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>linen_greatblade</t>
+        </is>
+      </c>
+      <c r="D86" s="3" t="inlineStr">
+        <is>
+          <t>weapon</t>
+        </is>
+      </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F86" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
+          <t>linen_cloth ×9
+wood_log ×6
+iron_ingot ×3</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>linen_tower_shield_recipe</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Tour en lin</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>linen_tower_shield</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>1</v>
+      </c>
+      <c r="G87" s="5" t="inlineStr">
+        <is>
+          <t>linen_cloth ×9
+wood_log ×9
+leather_strip ×3</t>
         </is>
       </c>
     </row>
@@ -7868,7 +9808,7 @@
         </is>
       </c>
       <c r="D2" s="3" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
@@ -7913,7 +9853,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E3" t="inlineStr">
         <is>
@@ -7958,7 +9898,7 @@
         </is>
       </c>
       <c r="D4" s="3" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
@@ -8003,7 +9943,7 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
@@ -8048,7 +9988,7 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
@@ -8421,10 +10361,1240 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P10"/>
+  <dimension ref="A1:P19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Nom</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Rareté</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Slot</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>2-mains</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Atk +</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>Def +</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>PV +</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>Crit chance +</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Crit dmg +</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Esquive +</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Vitesse +</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Regen +</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Prix vente</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Prix achat</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>wood_sword</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Épée en bois</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>Une arme basique pour débuter. Une main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>slime_blade</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Lame visqueuse</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>12</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>Une épée recouverte d'une étrange matière gélatineuse. Une main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>hunter_dagger</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Dague du chasseur</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>Une dague légère favorisant les coups précis. Une main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>gobelin_axe</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Hache gobeline</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J5" t="n">
+        <v>5</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M5" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" t="n">
+        <v>18</v>
+      </c>
+      <c r="O5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>Hache fruste taillée par les gobelins. Une main.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>two_handed_iron_sword</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Espadon de fer</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>Une longue lame qui demande de tenir des deux mains.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>iron_dagger</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Dague en fer</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>3</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>0</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="n">
+        <v>0</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>2</v>
+      </c>
+      <c r="M7" t="n">
+        <v>0</v>
+      </c>
+      <c r="N7" t="n">
+        <v>12</v>
+      </c>
+      <c r="O7" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>Dague affûtée, légère et discrète.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>goblin_blade</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Lame gobeline</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>uncommon</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="3" t="inlineStr">
+        <is>
+          <t>Lame ébréchée mais redoutable, taillée d'os de gobelin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>leather_main_droite</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Lame en cuir</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" t="n">
+        <v>1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>0</v>
+      </c>
+      <c r="I9" t="n">
+        <v>0</v>
+      </c>
+      <c r="J9" t="n">
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
+      <c r="M9" t="n">
+        <v>0</v>
+      </c>
+      <c r="N9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O9" t="n">
+        <v>12</v>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>Pièce de la panoplie leather — bonus de set actif dès 2 pièces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>linen_main_droite</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Lame en lin</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>Pièce de la panoplie linen — bonus de set actif dès 2 pièces.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>iron_sword</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Épée en fer</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>3</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>18</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Variante équilibrée de la dague en fer — atk + un peu de def/PV.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>iron_greatsword</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Espadon en fer</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>-5</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>-2</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>Lame à 2 mains — frappe lourde mais on s'expose en attaquant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>slime_morningstar</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Morningstar visqueuse</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>0</v>
+      </c>
+      <c r="J13" t="n">
+        <v>0</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>2</v>
+      </c>
+      <c r="N13" t="n">
+        <v>22</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Variante régen de la lame visqueuse — atk soutenue + un peu de régen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>slime_greatblade</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Lame visqueuse colossale</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>-4</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>-6</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>70</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>2 mains — frappe massive, on perd en résilience.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>gobelin_greataxe</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Grande hache gobeline</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>18</v>
+      </c>
+      <c r="G15" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J15" t="n">
+        <v>15</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>80</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>2 mains — crit massifs, on se découvre complètement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>leather_dagger</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Dague en cuir</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>Variante offensive de la lame en cuir — un peu d'attaque en plus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>leather_greatsword</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Grande lame en cuir</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>6</v>
+      </c>
+      <c r="G17" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>0</v>
+      </c>
+      <c r="K17" t="n">
+        <v>2</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>50</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>2 mains — atk solide pour la panoplie cuir, on perd en couverture.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>linen_rapier</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Rapière en lin</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="M18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P18" s="3" t="inlineStr">
+        <is>
+          <t>Variante speed/crit de la lame en lin — précise mais fragile.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>linen_greatblade</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Grande lame en lin</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" t="n">
+        <v>-3</v>
+      </c>
+      <c r="H19" t="n">
+        <v>0</v>
+      </c>
+      <c r="I19" t="n">
+        <v>3</v>
+      </c>
+      <c r="J19" t="n">
+        <v>6</v>
+      </c>
+      <c r="K19" t="n">
+        <v>-1</v>
+      </c>
+      <c r="L19" t="n">
+        <v>0</v>
+      </c>
+      <c r="M19" t="n">
+        <v>0</v>
+      </c>
+      <c r="N19" t="n">
+        <v>55</v>
+      </c>
+      <c r="O19" t="n">
+        <v>0</v>
+      </c>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>2 mains — crit dmg massif mais peu de couverture.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -8527,12 +11697,12 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>wood_sword</t>
+          <t>wooden_shield</t>
         </is>
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Épée en bois</t>
+          <t>Bouclier en bois</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -8542,7 +11712,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>main_droite</t>
+          <t>main_gauche</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -8551,13 +11721,13 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G2" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="G2" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="H2" s="3" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -8575,26 +11745,26 @@
         <v>0</v>
       </c>
       <c r="N2" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="O2" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>Une arme basique pour débuter. Une main.</t>
+          <t>Un bouclier léger, à porter en main gauche.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>slime_blade</t>
+          <t>iron_buckler</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Lame visqueuse</t>
+          <t>Rondache en fer</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -8604,7 +11774,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>main_droite</t>
+          <t>main_gauche</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -8613,13 +11783,13 @@
         </is>
       </c>
       <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
         <v>5</v>
       </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -8628,7 +11798,7 @@
         <v>0</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
         <v>0</v>
@@ -8637,26 +11807,26 @@
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>Une épée recouverte d'une étrange matière gélatineuse. Une main.</t>
+          <t>Un petit bouclier rond, à porter en main gauche.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>hunter_dagger</t>
+          <t>slime_shield</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Dague du chasseur</t>
+          <t>Bouclier visqueux</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
@@ -8666,7 +11836,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>main_droite</t>
+          <t>main_gauche</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -8675,16 +11845,16 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3" t="n">
         <v>0</v>
@@ -8699,36 +11869,36 @@
         <v>0</v>
       </c>
       <c r="N4" s="3" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="O4" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>Une dague légère favorisant les coups précis. Une main.</t>
+          <t>Bouclier en bois enveloppé de gel de slime — absorbe les chocs comme une éponge.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>gobelin_axe</t>
+          <t>leather_main_gauche</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Hache gobeline</t>
+          <t>Bouclier en cuir</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>uncommon</t>
+          <t>common</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>main_droite</t>
+          <t>main_gauche</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -8737,10 +11907,10 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -8749,10 +11919,10 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -8761,45 +11931,45 @@
         <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>18</v>
+        <v>4</v>
       </c>
       <c r="O5" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>Hache fruste taillée par les gobelins. Une main.</t>
+          <t>Pièce de la panoplie leather — bonus de set actif dès 2 pièces.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>two_handed_iron_sword</t>
+          <t>gobelin_main_gauche</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Espadon de fer</t>
+          <t>Bouclier gobelin</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>main_droite</t>
+          <t>main_gauche</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -8808,10 +11978,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -8823,26 +11993,26 @@
         <v>0</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>35</v>
+        <v>7</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>0</v>
+        <v>21</v>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Une longue lame qui demande de tenir des deux mains.</t>
+          <t>Pièce de la panoplie gobelin — bonus de set actif dès 2 pièces.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>iron_dagger</t>
+          <t>linen_main_gauche</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dague en fer</t>
+          <t>Bouclier en lin</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -8852,7 +12022,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>main_droite</t>
+          <t>main_gauche</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -8861,7 +12031,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -8870,46 +12040,46 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
+        <v>0</v>
+      </c>
+      <c r="J7" t="n">
         <v>2</v>
       </c>
-      <c r="J7" t="n">
-        <v>0</v>
-      </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
       </c>
       <c r="N7" t="n">
+        <v>4</v>
+      </c>
+      <c r="O7" t="n">
         <v>12</v>
       </c>
-      <c r="O7" t="n">
-        <v>0</v>
-      </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Dague affûtée, légère et discrète.</t>
+          <t>Pièce de la panoplie linen — bonus de set actif dès 2 pièces.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>goblin_blade</t>
+          <t>iron_warshield</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Lame gobeline</t>
+          <t>Pavois en fer</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>uncommon</t>
+          <t>common</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -8923,19 +12093,19 @@
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>0</v>
@@ -8947,31 +12117,31 @@
         <v>0</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>22</v>
+        <v>18</v>
       </c>
       <c r="O8" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Lame ébréchée mais redoutable, taillée d'os de gobelin.</t>
+          <t>Variante tanky de la rondache — plus de PV, moins d'esquive.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>leather_main_droite</t>
+          <t>iron_tower_shield</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lame en cuir</t>
+          <t>Tour en fer</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -8981,54 +12151,54 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
       </c>
       <c r="I9" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="J9" t="n">
         <v>0</v>
       </c>
       <c r="K9" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="L9" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>4</v>
+        <v>60</v>
       </c>
       <c r="O9" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Pièce de la panoplie leather — bonus de set actif dès 2 pièces.</t>
+          <t>Bouclier-tour à 2 mains — forteresse mobile au prix de l'offensive.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>linen_main_droite</t>
+          <t>slime_buckler</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Lame en lin</t>
+          <t>Bouclier de gel</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -9050,7 +12220,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>0</v>
@@ -9059,512 +12229,460 @@
         <v>0</v>
       </c>
       <c r="J10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="3" t="inlineStr">
+        <is>
+          <t>Variante régen du bouclier visqueux — moins de PV, plus de régen.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>slime_tower_shield</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Tour de gel</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>-5</v>
+      </c>
+      <c r="G11" t="n">
+        <v>12</v>
+      </c>
+      <c r="H11" t="n">
+        <v>18</v>
+      </c>
+      <c r="I11" t="n">
+        <v>0</v>
+      </c>
+      <c r="J11" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
+      <c r="M11" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" t="n">
+        <v>70</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>Bouclier 2 mains — pure défense, on n'attaque presque plus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_buckler</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Rondache gobeline</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="K10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="L10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M10" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N10" s="3" t="n">
+      <c r="J12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="3" t="inlineStr">
+        <is>
+          <t>Variante du bouclier gobelin — orientée crit + défense.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>gobelin_warshield</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pavois gobelin</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>-6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>9</v>
+      </c>
+      <c r="H13" t="n">
+        <v>0</v>
+      </c>
+      <c r="I13" t="n">
+        <v>5</v>
+      </c>
+      <c r="J13" t="n">
+        <v>-5</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" t="n">
+        <v>0</v>
+      </c>
+      <c r="N13" t="n">
+        <v>60</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>Bouclier gobelin 2 mains — défense brute + crit, on tape moins fort.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>leather_buckler</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Rondache en cuir</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>common</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>non</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H14" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="O10" s="3" t="n">
-        <v>12</v>
-      </c>
-      <c r="P10" s="3" t="inlineStr">
-        <is>
-          <t>Pièce de la panoplie linen — bonus de set actif dès 2 pièces.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:P7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="19" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
-    <col width="10" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="40" customWidth="1" min="16" max="16"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="2" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-      <c r="B1" s="2" t="inlineStr">
-        <is>
-          <t>Nom</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
-        <is>
-          <t>Rareté</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>Slot</t>
-        </is>
-      </c>
-      <c r="E1" s="2" t="inlineStr">
-        <is>
-          <t>2-mains</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
-        <is>
-          <t>Atk +</t>
-        </is>
-      </c>
-      <c r="G1" s="2" t="inlineStr">
-        <is>
-          <t>Def +</t>
-        </is>
-      </c>
-      <c r="H1" s="2" t="inlineStr">
-        <is>
-          <t>PV +</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>Crit chance +</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>Crit dmg +</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>Esquive +</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>Vitesse +</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>Regen +</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
-          <t>Prix vente</t>
-        </is>
-      </c>
-      <c r="O1" s="2" t="inlineStr">
-        <is>
-          <t>Prix achat</t>
-        </is>
-      </c>
-      <c r="P1" s="2" t="inlineStr">
-        <is>
-          <t>Description</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="3" t="inlineStr">
-        <is>
-          <t>wooden_shield</t>
-        </is>
-      </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Bouclier en bois</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="I14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="3" t="inlineStr">
+        <is>
+          <t>Variante tanky du bouclier en cuir — plus de PV, moins d'esquive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>leather_tower_shield</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Tour en cuir</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>-2</v>
+      </c>
+      <c r="G15" t="n">
+        <v>6</v>
+      </c>
+      <c r="H15" t="n">
+        <v>0</v>
+      </c>
+      <c r="I15" t="n">
+        <v>0</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
+        <v>3</v>
+      </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
+      <c r="M15" t="n">
+        <v>0</v>
+      </c>
+      <c r="N15" t="n">
+        <v>50</v>
+      </c>
+      <c r="O15" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>Bouclier 2 mains en cuir tanné — défense + esquive contre 0 attaque.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>linen_aegis</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Égide en lin</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>common</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
-        <is>
-          <t>main_gauche</t>
-        </is>
-      </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>non</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G2" s="3" t="n">
+      <c r="F16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="3" t="inlineStr">
+        <is>
+          <t>Variante esquive du bouclier en lin — optimisée pour les agiles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>linen_tower_shield</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Tour en lin</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>rare</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>oui</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" t="n">
         <v>3</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H17" t="n">
+        <v>0</v>
+      </c>
+      <c r="I17" t="n">
+        <v>0</v>
+      </c>
+      <c r="J17" t="n">
+        <v>-2</v>
+      </c>
+      <c r="K17" t="n">
         <v>5</v>
       </c>
-      <c r="I2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="O2" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P2" s="3" t="inlineStr">
-        <is>
-          <t>Un bouclier léger, à porter en main gauche.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>iron_buckler</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Rondache en fer</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>uncommon</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>main_gauche</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="F3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G3" t="n">
-        <v>5</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K3" t="n">
-        <v>2</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N3" t="n">
-        <v>14</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>Un petit bouclier rond, à porter en main gauche.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t>slime_shield</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>Bouclier visqueux</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
-        <is>
-          <t>uncommon</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>main_gauche</t>
-        </is>
-      </c>
-      <c r="E4" s="3" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="G4" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>6</v>
-      </c>
-      <c r="I4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N4" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="O4" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="3" t="inlineStr">
-        <is>
-          <t>Bouclier en bois enveloppé de gel de slime — absorbe les chocs comme une éponge.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>leather_main_gauche</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Bouclier en cuir</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>common</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>main_gauche</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="F5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" t="n">
-        <v>1</v>
-      </c>
-      <c r="H5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K5" t="n">
-        <v>1</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N5" t="n">
-        <v>4</v>
-      </c>
-      <c r="O5" t="n">
-        <v>12</v>
-      </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>Pièce de la panoplie leather — bonus de set actif dès 2 pièces.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t>gobelin_main_gauche</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>Bouclier gobelin</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
-        <is>
-          <t>uncommon</t>
-        </is>
-      </c>
-      <c r="D6" s="3" t="inlineStr">
-        <is>
-          <t>main_gauche</t>
-        </is>
-      </c>
-      <c r="E6" s="3" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="F6" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="G6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="O6" s="3" t="n">
-        <v>21</v>
-      </c>
-      <c r="P6" s="3" t="inlineStr">
-        <is>
-          <t>Pièce de la panoplie gobelin — bonus de set actif dès 2 pièces.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>linen_main_gauche</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Bouclier en lin</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>common</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>main_gauche</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>non</t>
-        </is>
-      </c>
-      <c r="F7" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" t="n">
-        <v>2</v>
-      </c>
-      <c r="K7" t="n">
-        <v>1</v>
-      </c>
-      <c r="L7" t="n">
-        <v>0</v>
-      </c>
-      <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="n">
-        <v>4</v>
-      </c>
-      <c r="O7" t="n">
-        <v>12</v>
-      </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>Pièce de la panoplie linen — bonus de set actif dès 2 pièces.</t>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
+      <c r="M17" t="n">
+        <v>0</v>
+      </c>
+      <c r="N17" t="n">
+        <v>55</v>
+      </c>
+      <c r="O17" t="n">
+        <v>0</v>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Bouclier 2 mains en lin — pure esquive, dégâts en chute libre.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Retire le doublon 'Espadon de fer' (legacy two_handed_iron_sword)
L'item legacy faisait doublon avec iron_greatsword (Espadon en fer) qui
appartient à la panoplie Fer (panoplie iron, +malus défensif).

- Retiré items.json + recette
- tuto.txt : remplace les exemples par iron_greatsword
- Régénère sakura_content.xlsx (23 feuilles)
- Nettoyage DB VPS : DELETE en cascade (2 inventaires + 1 def + 1 recette)
  avec backup pré-DELETE (lita_v2_backup_pre_legacy_sword_*.db)
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 2026-05-07 18:18 UTC</t>
+          <t>Généré le 2026-05-07 19:19 UTC</t>
         </is>
       </c>
     </row>
@@ -3398,7 +3398,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G87"/>
+  <dimension ref="A1:G86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -3952,27 +3952,27 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>two_handed_iron_sword_recipe</t>
+          <t>iron_helmet_recipe</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Espadon de fer</t>
+          <t>Casque de fer</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>two_handed_iron_sword</t>
+          <t>iron_helmet</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>helmet</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>main_droite</t>
+          <t>casque</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
@@ -3980,186 +3980,149 @@
       </c>
       <c r="G16" s="4" t="inlineStr">
         <is>
-          <t>iron_ingot ×8
-leather_strip ×2
-wood_log ×2</t>
+          <t>iron_ingot ×4
+leather_strip ×1</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>iron_helmet_recipe</t>
+          <t>iron_chest_recipe</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Casque de fer</t>
+          <t>Plastron de fer</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>iron_helmet</t>
+          <t>iron_chest</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>helmet</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>casque</t>
+          <t>plastron</t>
         </is>
       </c>
       <c r="F17" t="n">
         <v>1</v>
       </c>
       <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>iron_ingot ×6
+leather_strip ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>iron_legs_recipe</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Jambières de fer</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>iron_legs</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>legs</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>jambieres</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>iron_ingot ×5
+leather_strip ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>iron_boots_recipe</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Bottes en fer</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>iron_boots</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>boots</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>bottes</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
         <is>
           <t>iron_ingot ×4
 leather_strip ×1</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>iron_chest_recipe</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>Plastron de fer</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>iron_chest</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>chest</t>
-        </is>
-      </c>
-      <c r="E18" s="3" t="inlineStr">
-        <is>
-          <t>plastron</t>
-        </is>
-      </c>
-      <c r="F18" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
-        <is>
-          <t>iron_ingot ×6
-leather_strip ×2</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>iron_legs_recipe</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Jambières de fer</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>iron_legs</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>legs</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>jambieres</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>1</v>
-      </c>
-      <c r="G19" s="5" t="inlineStr">
-        <is>
-          <t>iron_ingot ×5
-leather_strip ×2</t>
-        </is>
-      </c>
-    </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>iron_boots_recipe</t>
+          <t>gobelin_crown_recipe</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Bottes en fer</t>
+          <t>Couronne gobeline</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>iron_boots</t>
+          <t>gobelin_crown</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>boots</t>
+          <t>helmet</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>bottes</t>
+          <t>casque</t>
         </is>
       </c>
       <c r="F20" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G20" s="4" t="inlineStr">
-        <is>
-          <t>iron_ingot ×4
-leather_strip ×1</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>gobelin_crown_recipe</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>Couronne gobeline</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>gobelin_crown</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>helmet</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>casque</t>
-        </is>
-      </c>
-      <c r="F21" t="n">
-        <v>1</v>
-      </c>
-      <c r="G21" s="5" t="inlineStr">
         <is>
           <t>gobelin_tooth ×6
 polished_stone ×2
@@ -4167,20 +4130,55 @@
         </is>
       </c>
     </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>iron_ring_recipe</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Anneau de fer</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>iron_ring</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>ring</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>bague</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>iron_ingot ×2</t>
+        </is>
+      </c>
+    </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>iron_ring_recipe</t>
+          <t>gobelin_ring_recipe</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Anneau de fer</t>
+          <t>Bague gobeline</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>iron_ring</t>
+          <t>gobelin_ring</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
@@ -4196,42 +4194,7 @@
       <c r="F22" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>iron_ingot ×2</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>gobelin_ring_recipe</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>Bague gobeline</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>gobelin_ring</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>ring</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>bague</t>
-        </is>
-      </c>
-      <c r="F23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G23" s="5" t="inlineStr">
+      <c r="G22" s="4" t="inlineStr">
         <is>
           <t>gobelin_tooth ×3
 iron_ingot ×1
@@ -4239,36 +4202,36 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
+    <row r="23">
+      <c r="A23" t="inlineStr">
         <is>
           <t>slime_pendant_recipe</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
+      <c r="B23" t="inlineStr">
         <is>
           <t>Pendentif de Slime</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>slime_pendant</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>necklace</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E23" t="inlineStr">
         <is>
           <t>collier</t>
         </is>
       </c>
-      <c r="F24" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="F23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
         <is>
           <t>slime_gel ×5
 polished_stone ×1
@@ -4276,30 +4239,66 @@
         </is>
       </c>
     </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>linen_hood_recipe</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Capuche en lin</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>linen_hood</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>helmet</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>casque</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
+          <t>linen_cloth ×4
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>linen_hood_recipe</t>
+          <t>linen_robe_recipe</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Capuche en lin</t>
+          <t>Robe en lin</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>linen_hood</t>
+          <t>linen_robe</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>helmet</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>casque</t>
+          <t>plastron</t>
         </is>
       </c>
       <c r="F25" t="n">
@@ -4307,7 +4306,7 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>linen_cloth ×4
+          <t>linen_cloth ×6
 leather_strip ×1</t>
         </is>
       </c>
@@ -4315,104 +4314,68 @@
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>linen_robe_recipe</t>
+          <t>linen_gloves_recipe</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Robe en lin</t>
+          <t>Mitaines en lin</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>linen_robe</t>
+          <t>linen_gloves</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>bracelet</t>
         </is>
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t>plastron</t>
+          <t>bracelet</t>
         </is>
       </c>
       <c r="F26" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G26" s="4" t="inlineStr">
-        <is>
-          <t>linen_cloth ×6
-leather_strip ×1</t>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>linen_cloth ×3</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>linen_gloves_recipe</t>
+          <t>slime_cloak_recipe</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Mitaines en lin</t>
+          <t>Cape gluante</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>linen_gloves</t>
+          <t>slime_cloak</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>bracelet</t>
+          <t>cape</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>bracelet</t>
+          <t>cape</t>
         </is>
       </c>
       <c r="F27" t="n">
         <v>1</v>
       </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>linen_cloth ×3</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="3" t="inlineStr">
-        <is>
-          <t>slime_cloak_recipe</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Cape gluante</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>slime_cloak</t>
-        </is>
-      </c>
-      <c r="D28" s="3" t="inlineStr">
-        <is>
-          <t>cape</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>cape</t>
-        </is>
-      </c>
-      <c r="F28" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
+      <c r="G27" s="5" t="inlineStr">
         <is>
           <t>slime_gel ×5
 linen_cloth ×3
@@ -4420,36 +4383,36 @@
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>goblin_amulet_recipe</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="B28" s="3" t="inlineStr">
         <is>
           <t>Amulette gobeline</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
+      <c r="C28" s="3" t="inlineStr">
         <is>
           <t>goblin_amulet</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr">
+      <c r="D28" s="3" t="inlineStr">
         <is>
           <t>necklace</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr">
+      <c r="E28" s="3" t="inlineStr">
         <is>
           <t>collier</t>
         </is>
       </c>
-      <c r="F29" t="n">
-        <v>1</v>
-      </c>
-      <c r="G29" s="5" t="inlineStr">
+      <c r="F28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G28" s="4" t="inlineStr">
         <is>
           <t>gobelin_tooth ×5
 polished_stone ×2
@@ -4457,107 +4420,107 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>polished_stone_ring_recipe</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Anneau de pierre polie</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>polished_stone_ring</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>ring</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>bague</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>1</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>polished_stone ×3</t>
+        </is>
+      </c>
+    </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>polished_stone_ring_recipe</t>
+          <t>iron_gauntlets_recipe</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>Anneau de pierre polie</t>
+          <t>Gantelets en fer</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>polished_stone_ring</t>
+          <t>iron_gauntlets</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>ring</t>
+          <t>bracelet</t>
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr">
         <is>
-          <t>bague</t>
+          <t>bracelet</t>
         </is>
       </c>
       <c r="F30" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>polished_stone ×3</t>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>iron_ingot ×4
+leather_strip ×2</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>iron_gauntlets_recipe</t>
+          <t>iron_dagger_recipe</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Gantelets en fer</t>
+          <t>Dague en fer</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>iron_gauntlets</t>
+          <t>iron_dagger</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>bracelet</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>bracelet</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="F31" t="n">
         <v>1</v>
       </c>
       <c r="G31" s="5" t="inlineStr">
-        <is>
-          <t>iron_ingot ×4
-leather_strip ×2</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
-        <is>
-          <t>iron_dagger_recipe</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>Dague en fer</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>iron_dagger</t>
-        </is>
-      </c>
-      <c r="D32" s="3" t="inlineStr">
-        <is>
-          <t>weapon</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>main_droite</t>
-        </is>
-      </c>
-      <c r="F32" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>iron_ingot ×2
 wood_log ×1
@@ -4565,36 +4528,36 @@
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>goblin_blade_recipe</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="B32" s="3" t="inlineStr">
         <is>
           <t>Lame gobeline</t>
         </is>
       </c>
-      <c r="C33" t="inlineStr">
+      <c r="C32" s="3" t="inlineStr">
         <is>
           <t>goblin_blade</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr">
+      <c r="D32" s="3" t="inlineStr">
         <is>
           <t>weapon</t>
         </is>
       </c>
-      <c r="E33" t="inlineStr">
+      <c r="E32" s="3" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F33" t="n">
-        <v>1</v>
-      </c>
-      <c r="G33" s="5" t="inlineStr">
+      <c r="F32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="4" t="inlineStr">
         <is>
           <t>gobelin_tooth ×4
 iron_ingot ×2
@@ -4602,36 +4565,36 @@
         </is>
       </c>
     </row>
-    <row r="34">
-      <c r="A34" s="3" t="inlineStr">
+    <row r="33">
+      <c r="A33" t="inlineStr">
         <is>
           <t>slime_shield_recipe</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
+      <c r="B33" t="inlineStr">
         <is>
           <t>Bouclier visqueux</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>slime_shield</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D33" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E33" t="inlineStr">
         <is>
           <t>main_gauche</t>
         </is>
       </c>
-      <c r="F34" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="F33" t="n">
+        <v>1</v>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
         <is>
           <t>slime_gel ×4
 wood_log ×3
@@ -4639,36 +4602,36 @@
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>gobelin_plastron_recipe</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="B34" s="3" t="inlineStr">
         <is>
           <t>Plastron gobelin</t>
         </is>
       </c>
-      <c r="C35" t="inlineStr">
+      <c r="C34" s="3" t="inlineStr">
         <is>
           <t>gobelin_plastron</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr">
+      <c r="D34" s="3" t="inlineStr">
         <is>
           <t>chest</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr">
+      <c r="E34" s="3" t="inlineStr">
         <is>
           <t>plastron</t>
         </is>
       </c>
-      <c r="F35" t="n">
-        <v>1</v>
-      </c>
-      <c r="G35" s="5" t="inlineStr">
+      <c r="F34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
         <is>
           <t>gobelin_tooth ×5
 iron_ingot ×2
@@ -4676,36 +4639,36 @@
         </is>
       </c>
     </row>
-    <row r="36">
-      <c r="A36" s="3" t="inlineStr">
+    <row r="35">
+      <c r="A35" t="inlineStr">
         <is>
           <t>gobelin_jambieres_recipe</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t>Jambières gobelin</t>
         </is>
       </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>gobelin_jambieres</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D35" t="inlineStr">
         <is>
           <t>legs</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E35" t="inlineStr">
         <is>
           <t>jambieres</t>
         </is>
       </c>
-      <c r="F36" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G36" s="4" t="inlineStr">
+      <c r="F35" t="n">
+        <v>1</v>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
         <is>
           <t>gobelin_tooth ×4
 iron_ingot ×2
@@ -4713,36 +4676,36 @@
         </is>
       </c>
     </row>
-    <row r="37">
-      <c r="A37" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
         <is>
           <t>gobelin_bottes_recipe</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="B36" s="3" t="inlineStr">
         <is>
           <t>Bottes gobelin</t>
         </is>
       </c>
-      <c r="C37" t="inlineStr">
+      <c r="C36" s="3" t="inlineStr">
         <is>
           <t>gobelin_bottes</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr">
+      <c r="D36" s="3" t="inlineStr">
         <is>
           <t>boots</t>
         </is>
       </c>
-      <c r="E37" t="inlineStr">
+      <c r="E36" s="3" t="inlineStr">
         <is>
           <t>bottes</t>
         </is>
       </c>
-      <c r="F37" t="n">
-        <v>1</v>
-      </c>
-      <c r="G37" s="5" t="inlineStr">
+      <c r="F36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G36" s="4" t="inlineStr">
         <is>
           <t>gobelin_tooth ×3
 iron_ingot ×1
@@ -4750,36 +4713,36 @@
         </is>
       </c>
     </row>
-    <row r="38">
-      <c r="A38" s="3" t="inlineStr">
+    <row r="37">
+      <c r="A37" t="inlineStr">
         <is>
           <t>gobelin_main_gauche_recipe</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B37" t="inlineStr">
         <is>
           <t>Bouclier gobelin</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>gobelin_main_gauche</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D37" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E37" t="inlineStr">
         <is>
           <t>main_gauche</t>
         </is>
       </c>
-      <c r="F38" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G38" s="4" t="inlineStr">
+      <c r="F37" t="n">
+        <v>1</v>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
         <is>
           <t>gobelin_tooth ×3
 iron_ingot ×1
@@ -4788,72 +4751,72 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_bracelet_recipe</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Bracelet gobelin</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>gobelin_bracelet</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>bracelet</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>bracelet</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×2
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>gobelin_bracelet_recipe</t>
+          <t>gobelin_ceinture_recipe</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Bracelet gobelin</t>
+          <t>Ceinture gobelin</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>gobelin_bracelet</t>
+          <t>gobelin_ceinture</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>bracelet</t>
+          <t>belt</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>bracelet</t>
+          <t>ceinture</t>
         </is>
       </c>
       <c r="F39" t="n">
         <v>1</v>
       </c>
       <c r="G39" s="5" t="inlineStr">
-        <is>
-          <t>gobelin_tooth ×2
-iron_ingot ×1</t>
-        </is>
-      </c>
-    </row>
-    <row r="40">
-      <c r="A40" s="3" t="inlineStr">
-        <is>
-          <t>gobelin_ceinture_recipe</t>
-        </is>
-      </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>Ceinture gobelin</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
-        <is>
-          <t>gobelin_ceinture</t>
-        </is>
-      </c>
-      <c r="D40" s="3" t="inlineStr">
-        <is>
-          <t>belt</t>
-        </is>
-      </c>
-      <c r="E40" s="3" t="inlineStr">
-        <is>
-          <t>ceinture</t>
-        </is>
-      </c>
-      <c r="F40" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>gobelin_tooth ×2
 iron_ingot ×1
@@ -4861,36 +4824,36 @@
         </is>
       </c>
     </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
         <is>
           <t>gobelin_cape_recipe</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="B40" s="3" t="inlineStr">
         <is>
           <t>Cape gobelin</t>
         </is>
       </c>
-      <c r="C41" t="inlineStr">
+      <c r="C40" s="3" t="inlineStr">
         <is>
           <t>gobelin_cape</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr">
+      <c r="D40" s="3" t="inlineStr">
         <is>
           <t>cape</t>
         </is>
       </c>
-      <c r="E41" t="inlineStr">
+      <c r="E40" s="3" t="inlineStr">
         <is>
           <t>cape</t>
         </is>
       </c>
-      <c r="F41" t="n">
-        <v>1</v>
-      </c>
-      <c r="G41" s="5" t="inlineStr">
+      <c r="F40" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G40" s="4" t="inlineStr">
         <is>
           <t>gobelin_tooth ×4
 linen_cloth ×2
@@ -4898,72 +4861,72 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>gobelin_boucle_oreille_recipe</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Boucle gobelin</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>gobelin_boucle_oreille</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>earring</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>boucle_oreille</t>
+        </is>
+      </c>
+      <c r="F41" t="n">
+        <v>1</v>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>gobelin_tooth ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>gobelin_boucle_oreille_recipe</t>
+          <t>iron_collier_recipe</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Boucle gobelin</t>
+          <t>Collier en fer</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>gobelin_boucle_oreille</t>
+          <t>iron_collier</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>earring</t>
+          <t>necklace</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
         <is>
-          <t>boucle_oreille</t>
+          <t>collier</t>
         </is>
       </c>
       <c r="F42" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G42" s="4" t="inlineStr">
-        <is>
-          <t>gobelin_tooth ×2
-polished_stone ×1</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" t="inlineStr">
-        <is>
-          <t>iron_collier_recipe</t>
-        </is>
-      </c>
-      <c r="B43" t="inlineStr">
-        <is>
-          <t>Collier en fer</t>
-        </is>
-      </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>iron_collier</t>
-        </is>
-      </c>
-      <c r="D43" t="inlineStr">
-        <is>
-          <t>necklace</t>
-        </is>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>collier</t>
-        </is>
-      </c>
-      <c r="F43" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" s="5" t="inlineStr">
         <is>
           <t>iron_ingot ×4
 polished_stone ×1
@@ -4971,72 +4934,72 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>iron_ceinture_recipe</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Ceinture en fer</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>iron_ceinture</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>belt</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>ceinture</t>
+        </is>
+      </c>
+      <c r="F43" t="n">
+        <v>1</v>
+      </c>
+      <c r="G43" s="5" t="inlineStr">
+        <is>
+          <t>iron_ingot ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>iron_ceinture_recipe</t>
+          <t>iron_cape_recipe</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>Ceinture en fer</t>
+          <t>Cape en fer</t>
         </is>
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>iron_ceinture</t>
+          <t>iron_cape</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>belt</t>
+          <t>cape</t>
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>ceinture</t>
+          <t>cape</t>
         </is>
       </c>
       <c r="F44" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G44" s="4" t="inlineStr">
-        <is>
-          <t>iron_ingot ×2
-leather_strip ×1</t>
-        </is>
-      </c>
-    </row>
-    <row r="45">
-      <c r="A45" t="inlineStr">
-        <is>
-          <t>iron_cape_recipe</t>
-        </is>
-      </c>
-      <c r="B45" t="inlineStr">
-        <is>
-          <t>Cape en fer</t>
-        </is>
-      </c>
-      <c r="C45" t="inlineStr">
-        <is>
-          <t>iron_cape</t>
-        </is>
-      </c>
-      <c r="D45" t="inlineStr">
-        <is>
-          <t>cape</t>
-        </is>
-      </c>
-      <c r="E45" t="inlineStr">
-        <is>
-          <t>cape</t>
-        </is>
-      </c>
-      <c r="F45" t="n">
-        <v>1</v>
-      </c>
-      <c r="G45" s="5" t="inlineStr">
         <is>
           <t>iron_ingot ×4
 linen_cloth ×2
@@ -5044,72 +5007,72 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>iron_boucle_oreille_recipe</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Boucle en fer</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>iron_boucle_oreille</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>earring</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>boucle_oreille</t>
+        </is>
+      </c>
+      <c r="F45" t="n">
+        <v>1</v>
+      </c>
+      <c r="G45" s="5" t="inlineStr">
+        <is>
+          <t>iron_ingot ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
     <row r="46">
       <c r="A46" s="3" t="inlineStr">
         <is>
-          <t>iron_boucle_oreille_recipe</t>
+          <t>leather_main_droite_recipe</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>Boucle en fer</t>
+          <t>Lame en cuir</t>
         </is>
       </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
-          <t>iron_boucle_oreille</t>
+          <t>leather_main_droite</t>
         </is>
       </c>
       <c r="D46" s="3" t="inlineStr">
         <is>
-          <t>earring</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>boucle_oreille</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="F46" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G46" s="4" t="inlineStr">
-        <is>
-          <t>iron_ingot ×2
-polished_stone ×1</t>
-        </is>
-      </c>
-    </row>
-    <row r="47">
-      <c r="A47" t="inlineStr">
-        <is>
-          <t>leather_main_droite_recipe</t>
-        </is>
-      </c>
-      <c r="B47" t="inlineStr">
-        <is>
-          <t>Lame en cuir</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>leather_main_droite</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>weapon</t>
-        </is>
-      </c>
-      <c r="E47" t="inlineStr">
-        <is>
-          <t>main_droite</t>
-        </is>
-      </c>
-      <c r="F47" t="n">
-        <v>1</v>
-      </c>
-      <c r="G47" s="5" t="inlineStr">
         <is>
           <t>leather_strip ×3
 wood_log ×2
@@ -5117,36 +5080,36 @@
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="3" t="inlineStr">
+    <row r="47">
+      <c r="A47" t="inlineStr">
         <is>
           <t>leather_main_gauche_recipe</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B47" t="inlineStr">
         <is>
           <t>Bouclier en cuir</t>
         </is>
       </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C47" t="inlineStr">
         <is>
           <t>leather_main_gauche</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="D47" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E47" t="inlineStr">
         <is>
           <t>main_gauche</t>
         </is>
       </c>
-      <c r="F48" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G48" s="4" t="inlineStr">
+      <c r="F47" t="n">
+        <v>1</v>
+      </c>
+      <c r="G47" s="5" t="inlineStr">
         <is>
           <t>leather_strip ×3
 wood_log ×3
@@ -5154,36 +5117,36 @@
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" t="inlineStr">
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
         <is>
           <t>leather_collier_recipe</t>
         </is>
       </c>
-      <c r="B49" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>Collier en cuir</t>
         </is>
       </c>
-      <c r="C49" t="inlineStr">
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>leather_collier</t>
         </is>
       </c>
-      <c r="D49" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>necklace</t>
         </is>
       </c>
-      <c r="E49" t="inlineStr">
+      <c r="E48" s="3" t="inlineStr">
         <is>
           <t>collier</t>
         </is>
       </c>
-      <c r="F49" t="n">
-        <v>1</v>
-      </c>
-      <c r="G49" s="5" t="inlineStr">
+      <c r="F48" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G48" s="4" t="inlineStr">
         <is>
           <t>leather_strip ×4
 polished_stone ×1
@@ -5191,102 +5154,138 @@
         </is>
       </c>
     </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>leather_bague_recipe</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Bague en cuir</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>leather_bague</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>ring</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>bague</t>
+        </is>
+      </c>
+      <c r="F49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G49" s="5" t="inlineStr">
+        <is>
+          <t>leather_strip ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
     <row r="50">
       <c r="A50" s="3" t="inlineStr">
         <is>
-          <t>leather_bague_recipe</t>
+          <t>leather_cape_recipe</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>Bague en cuir</t>
+          <t>Cape en cuir</t>
         </is>
       </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
-          <t>leather_bague</t>
+          <t>leather_cape</t>
         </is>
       </c>
       <c r="D50" s="3" t="inlineStr">
         <is>
-          <t>ring</t>
+          <t>cape</t>
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr">
         <is>
-          <t>bague</t>
+          <t>cape</t>
         </is>
       </c>
       <c r="F50" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G50" s="4" t="inlineStr">
+        <is>
+          <t>leather_strip ×5
+linen_cloth ×2</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>leather_boucle_oreille_recipe</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Boucle en cuir</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>leather_boucle_oreille</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>earring</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>boucle_oreille</t>
+        </is>
+      </c>
+      <c r="F51" t="n">
+        <v>1</v>
+      </c>
+      <c r="G51" s="5" t="inlineStr">
         <is>
           <t>leather_strip ×2
 polished_stone ×1</t>
         </is>
       </c>
     </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>leather_cape_recipe</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>Cape en cuir</t>
-        </is>
-      </c>
-      <c r="C51" t="inlineStr">
-        <is>
-          <t>leather_cape</t>
-        </is>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>cape</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>cape</t>
-        </is>
-      </c>
-      <c r="F51" t="n">
-        <v>1</v>
-      </c>
-      <c r="G51" s="5" t="inlineStr">
-        <is>
-          <t>leather_strip ×5
-linen_cloth ×2</t>
-        </is>
-      </c>
-    </row>
     <row r="52">
       <c r="A52" s="3" t="inlineStr">
         <is>
-          <t>leather_boucle_oreille_recipe</t>
+          <t>linen_jambieres_recipe</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>Boucle en cuir</t>
+          <t>Jambières en lin</t>
         </is>
       </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
-          <t>leather_boucle_oreille</t>
+          <t>linen_jambieres</t>
         </is>
       </c>
       <c r="D52" s="3" t="inlineStr">
         <is>
-          <t>earring</t>
+          <t>legs</t>
         </is>
       </c>
       <c r="E52" s="3" t="inlineStr">
         <is>
-          <t>boucle_oreille</t>
+          <t>jambieres</t>
         </is>
       </c>
       <c r="F52" s="3" t="n">
@@ -5294,35 +5293,35 @@
       </c>
       <c r="G52" s="4" t="inlineStr">
         <is>
-          <t>leather_strip ×2
-polished_stone ×1</t>
+          <t>linen_cloth ×4
+leather_strip ×2</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>linen_jambieres_recipe</t>
+          <t>linen_bottes_recipe</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Jambières en lin</t>
+          <t>Bottes en lin</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>linen_jambieres</t>
+          <t>linen_bottes</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>legs</t>
+          <t>boots</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>jambieres</t>
+          <t>bottes</t>
         </is>
       </c>
       <c r="F53" t="n">
@@ -5330,77 +5329,41 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>linen_cloth ×4
-leather_strip ×2</t>
+          <t>linen_cloth ×3
+leather_strip ×1</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="3" t="inlineStr">
         <is>
-          <t>linen_bottes_recipe</t>
+          <t>linen_main_droite_recipe</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>Bottes en lin</t>
+          <t>Lame en lin</t>
         </is>
       </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
-          <t>linen_bottes</t>
+          <t>linen_main_droite</t>
         </is>
       </c>
       <c r="D54" s="3" t="inlineStr">
         <is>
-          <t>boots</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr">
         <is>
-          <t>bottes</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="F54" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G54" s="4" t="inlineStr">
-        <is>
-          <t>linen_cloth ×3
-leather_strip ×1</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>linen_main_droite_recipe</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>Lame en lin</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>linen_main_droite</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>weapon</t>
-        </is>
-      </c>
-      <c r="E55" t="inlineStr">
-        <is>
-          <t>main_droite</t>
-        </is>
-      </c>
-      <c r="F55" t="n">
-        <v>1</v>
-      </c>
-      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>linen_cloth ×3
 wood_log ×2
@@ -5408,36 +5371,36 @@
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+    <row r="55">
+      <c r="A55" t="inlineStr">
         <is>
           <t>linen_main_gauche_recipe</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
+      <c r="B55" t="inlineStr">
         <is>
           <t>Bouclier en lin</t>
         </is>
       </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C55" t="inlineStr">
         <is>
           <t>linen_main_gauche</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D55" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E55" t="inlineStr">
         <is>
           <t>main_gauche</t>
         </is>
       </c>
-      <c r="F56" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G56" s="4" t="inlineStr">
+      <c r="F55" t="n">
+        <v>1</v>
+      </c>
+      <c r="G55" s="5" t="inlineStr">
         <is>
           <t>linen_cloth ×3
 wood_log ×3
@@ -5445,36 +5408,36 @@
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>linen_collier_recipe</t>
         </is>
       </c>
-      <c r="B57" t="inlineStr">
+      <c r="B56" s="3" t="inlineStr">
         <is>
           <t>Collier en lin</t>
         </is>
       </c>
-      <c r="C57" t="inlineStr">
+      <c r="C56" s="3" t="inlineStr">
         <is>
           <t>linen_collier</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
+      <c r="D56" s="3" t="inlineStr">
         <is>
           <t>necklace</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr">
+      <c r="E56" s="3" t="inlineStr">
         <is>
           <t>collier</t>
         </is>
       </c>
-      <c r="F57" t="n">
-        <v>1</v>
-      </c>
-      <c r="G57" s="5" t="inlineStr">
+      <c r="F56" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G56" s="4" t="inlineStr">
         <is>
           <t>linen_cloth ×4
 polished_stone ×1
@@ -5482,102 +5445,138 @@
         </is>
       </c>
     </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>linen_bague_recipe</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>Bague en lin</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>linen_bague</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ring</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>bague</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>1</v>
+      </c>
+      <c r="G57" s="5" t="inlineStr">
+        <is>
+          <t>linen_cloth ×2
+polished_stone ×1</t>
+        </is>
+      </c>
+    </row>
     <row r="58">
       <c r="A58" s="3" t="inlineStr">
         <is>
-          <t>linen_bague_recipe</t>
+          <t>linen_ceinture_recipe</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Bague en lin</t>
+          <t>Ceinture en lin</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>linen_bague</t>
+          <t>linen_ceinture</t>
         </is>
       </c>
       <c r="D58" s="3" t="inlineStr">
         <is>
-          <t>ring</t>
+          <t>belt</t>
         </is>
       </c>
       <c r="E58" s="3" t="inlineStr">
         <is>
-          <t>bague</t>
+          <t>ceinture</t>
         </is>
       </c>
       <c r="F58" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G58" s="4" t="inlineStr">
+        <is>
+          <t>linen_cloth ×2
+iron_ingot ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>linen_boucle_oreille_recipe</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>Boucle en lin</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>linen_boucle_oreille</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>earring</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>boucle_oreille</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>1</v>
+      </c>
+      <c r="G59" s="5" t="inlineStr">
         <is>
           <t>linen_cloth ×2
 polished_stone ×1</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>linen_ceinture_recipe</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>Ceinture en lin</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>linen_ceinture</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>belt</t>
-        </is>
-      </c>
-      <c r="E59" t="inlineStr">
-        <is>
-          <t>ceinture</t>
-        </is>
-      </c>
-      <c r="F59" t="n">
-        <v>1</v>
-      </c>
-      <c r="G59" s="5" t="inlineStr">
-        <is>
-          <t>linen_cloth ×2
-iron_ingot ×1</t>
-        </is>
-      </c>
-    </row>
     <row r="60">
       <c r="A60" s="3" t="inlineStr">
         <is>
-          <t>linen_boucle_oreille_recipe</t>
+          <t>slime_casque_recipe</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>Boucle en lin</t>
+          <t>Casque de slime</t>
         </is>
       </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
-          <t>linen_boucle_oreille</t>
+          <t>slime_casque</t>
         </is>
       </c>
       <c r="D60" s="3" t="inlineStr">
         <is>
-          <t>earring</t>
+          <t>helmet</t>
         </is>
       </c>
       <c r="E60" s="3" t="inlineStr">
         <is>
-          <t>boucle_oreille</t>
+          <t>casque</t>
         </is>
       </c>
       <c r="F60" s="3" t="n">
@@ -5585,35 +5584,35 @@
       </c>
       <c r="G60" s="4" t="inlineStr">
         <is>
-          <t>linen_cloth ×2
-polished_stone ×1</t>
+          <t>slime_gel ×4
+leather_strip ×1</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>slime_casque_recipe</t>
+          <t>slime_plastron_recipe</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Casque de slime</t>
+          <t>Plastron de slime</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>slime_casque</t>
+          <t>slime_plastron</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>helmet</t>
+          <t>chest</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>casque</t>
+          <t>plastron</t>
         </is>
       </c>
       <c r="F61" t="n">
@@ -5621,35 +5620,35 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>slime_gel ×4
-leather_strip ×1</t>
+          <t>slime_gel ×5
+leather_strip ×2</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="3" t="inlineStr">
         <is>
-          <t>slime_plastron_recipe</t>
+          <t>slime_jambieres_recipe</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Plastron de slime</t>
+          <t>Jambières de slime</t>
         </is>
       </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
-          <t>slime_plastron</t>
+          <t>slime_jambieres</t>
         </is>
       </c>
       <c r="D62" s="3" t="inlineStr">
         <is>
-          <t>chest</t>
+          <t>legs</t>
         </is>
       </c>
       <c r="E62" s="3" t="inlineStr">
         <is>
-          <t>plastron</t>
+          <t>jambieres</t>
         </is>
       </c>
       <c r="F62" s="3" t="n">
@@ -5657,7 +5656,7 @@
       </c>
       <c r="G62" s="4" t="inlineStr">
         <is>
-          <t>slime_gel ×5
+          <t>slime_gel ×4
 leather_strip ×2</t>
         </is>
       </c>
@@ -5665,27 +5664,27 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>slime_jambieres_recipe</t>
+          <t>slime_bottes_recipe</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Jambières de slime</t>
+          <t>Bottes de slime</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>slime_jambieres</t>
+          <t>slime_bottes</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>legs</t>
+          <t>boots</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>jambieres</t>
+          <t>bottes</t>
         </is>
       </c>
       <c r="F63" t="n">
@@ -5693,35 +5692,35 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>slime_gel ×4
-leather_strip ×2</t>
+          <t>slime_gel ×3
+leather_strip ×1</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="3" t="inlineStr">
         <is>
-          <t>slime_bottes_recipe</t>
+          <t>slime_bracelet_recipe</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Bottes de slime</t>
+          <t>Bracelet de slime</t>
         </is>
       </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
-          <t>slime_bottes</t>
+          <t>slime_bracelet</t>
         </is>
       </c>
       <c r="D64" s="3" t="inlineStr">
         <is>
-          <t>boots</t>
+          <t>bracelet</t>
         </is>
       </c>
       <c r="E64" s="3" t="inlineStr">
         <is>
-          <t>bottes</t>
+          <t>bracelet</t>
         </is>
       </c>
       <c r="F64" s="3" t="n">
@@ -5729,35 +5728,35 @@
       </c>
       <c r="G64" s="4" t="inlineStr">
         <is>
-          <t>slime_gel ×3
-leather_strip ×1</t>
+          <t>slime_gel ×2
+iron_ingot ×1</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>slime_bracelet_recipe</t>
+          <t>slime_bague_recipe</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Bracelet de slime</t>
+          <t>Bague de slime</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>slime_bracelet</t>
+          <t>slime_bague</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>bracelet</t>
+          <t>ring</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>bracelet</t>
+          <t>bague</t>
         </is>
       </c>
       <c r="F65" t="n">
@@ -5766,148 +5765,112 @@
       <c r="G65" s="5" t="inlineStr">
         <is>
           <t>slime_gel ×2
-iron_ingot ×1</t>
+polished_stone ×1</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="3" t="inlineStr">
         <is>
-          <t>slime_bague_recipe</t>
+          <t>slime_ceinture_recipe</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Bague de slime</t>
+          <t>Ceinture de slime</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>slime_bague</t>
+          <t>slime_ceinture</t>
         </is>
       </c>
       <c r="D66" s="3" t="inlineStr">
         <is>
-          <t>ring</t>
+          <t>belt</t>
         </is>
       </c>
       <c r="E66" s="3" t="inlineStr">
         <is>
-          <t>bague</t>
+          <t>ceinture</t>
         </is>
       </c>
       <c r="F66" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G66" s="4" t="inlineStr">
+        <is>
+          <t>slime_gel ×2
+leather_strip ×1</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>slime_boucle_oreille_recipe</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Boucle de slime</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>slime_boucle_oreille</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>earring</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>boucle_oreille</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>1</v>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
         <is>
           <t>slime_gel ×2
 polished_stone ×1</t>
         </is>
       </c>
     </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>slime_ceinture_recipe</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>Ceinture de slime</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>slime_ceinture</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>belt</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>ceinture</t>
-        </is>
-      </c>
-      <c r="F67" t="n">
-        <v>1</v>
-      </c>
-      <c r="G67" s="5" t="inlineStr">
-        <is>
-          <t>slime_gel ×2
-leather_strip ×1</t>
-        </is>
-      </c>
-    </row>
     <row r="68">
       <c r="A68" s="3" t="inlineStr">
         <is>
-          <t>slime_boucle_oreille_recipe</t>
+          <t>iron_sword_recipe</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
         <is>
-          <t>Boucle de slime</t>
+          <t>Épée en fer</t>
         </is>
       </c>
       <c r="C68" s="3" t="inlineStr">
         <is>
-          <t>slime_boucle_oreille</t>
+          <t>iron_sword</t>
         </is>
       </c>
       <c r="D68" s="3" t="inlineStr">
         <is>
-          <t>earring</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="E68" s="3" t="inlineStr">
         <is>
-          <t>boucle_oreille</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="F68" s="3" t="n">
         <v>1</v>
       </c>
       <c r="G68" s="4" t="inlineStr">
-        <is>
-          <t>slime_gel ×2
-polished_stone ×1</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>iron_sword_recipe</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>Épée en fer</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>iron_sword</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
-        <is>
-          <t>weapon</t>
-        </is>
-      </c>
-      <c r="E69" t="inlineStr">
-        <is>
-          <t>main_droite</t>
-        </is>
-      </c>
-      <c r="F69" t="n">
-        <v>1</v>
-      </c>
-      <c r="G69" s="5" t="inlineStr">
         <is>
           <t>iron_ingot ×3
 wood_log ×1
@@ -5915,25 +5878,61 @@
         </is>
       </c>
     </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>iron_warshield_recipe</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Pavois en fer</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>iron_warshield</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>1</v>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>iron_ingot ×4
+leather_strip ×2</t>
+        </is>
+      </c>
+    </row>
     <row r="70">
       <c r="A70" s="3" t="inlineStr">
         <is>
-          <t>iron_warshield_recipe</t>
+          <t>iron_greatsword_recipe</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Pavois en fer</t>
+          <t>Espadon en fer</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>iron_warshield</t>
+          <t>iron_greatsword</t>
         </is>
       </c>
       <c r="D70" s="3" t="inlineStr">
         <is>
-          <t>shield</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="E70" s="3" t="inlineStr">
@@ -5945,42 +5944,6 @@
         <v>1</v>
       </c>
       <c r="G70" s="4" t="inlineStr">
-        <is>
-          <t>iron_ingot ×4
-leather_strip ×2</t>
-        </is>
-      </c>
-    </row>
-    <row r="71">
-      <c r="A71" t="inlineStr">
-        <is>
-          <t>iron_greatsword_recipe</t>
-        </is>
-      </c>
-      <c r="B71" t="inlineStr">
-        <is>
-          <t>Espadon en fer</t>
-        </is>
-      </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>iron_greatsword</t>
-        </is>
-      </c>
-      <c r="D71" t="inlineStr">
-        <is>
-          <t>weapon</t>
-        </is>
-      </c>
-      <c r="E71" t="inlineStr">
-        <is>
-          <t>main_droite</t>
-        </is>
-      </c>
-      <c r="F71" t="n">
-        <v>1</v>
-      </c>
-      <c r="G71" s="5" t="inlineStr">
         <is>
           <t>iron_ingot ×6
 wood_log ×3
@@ -5988,25 +5951,61 @@
         </is>
       </c>
     </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>iron_tower_shield_recipe</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Tour en fer</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>iron_tower_shield</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>shield</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>main_droite</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="5" t="inlineStr">
+        <is>
+          <t>iron_ingot ×9
+leather_strip ×3</t>
+        </is>
+      </c>
+    </row>
     <row r="72">
       <c r="A72" s="3" t="inlineStr">
         <is>
-          <t>iron_tower_shield_recipe</t>
+          <t>slime_morningstar_recipe</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Tour en fer</t>
+          <t>Morningstar visqueuse</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
         <is>
-          <t>iron_tower_shield</t>
+          <t>slime_morningstar</t>
         </is>
       </c>
       <c r="D72" s="3" t="inlineStr">
         <is>
-          <t>shield</t>
+          <t>weapon</t>
         </is>
       </c>
       <c r="E72" s="3" t="inlineStr">
@@ -6019,30 +6018,30 @@
       </c>
       <c r="G72" s="4" t="inlineStr">
         <is>
-          <t>iron_ingot ×9
-leather_strip ×3</t>
+          <t>slime_gel ×3
+wood_log ×2</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>slime_morningstar_recipe</t>
+          <t>slime_buckler_recipe</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Morningstar visqueuse</t>
+          <t>Bouclier de gel</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>slime_morningstar</t>
+          <t>slime_buckler</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>weapon</t>
+          <t>shield</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -6054,42 +6053,6 @@
         <v>1</v>
       </c>
       <c r="G73" s="5" t="inlineStr">
-        <is>
-          <t>slime_gel ×3
-wood_log ×2</t>
-        </is>
-      </c>
-    </row>
-    <row r="74">
-      <c r="A74" s="3" t="inlineStr">
-        <is>
-          <t>slime_buckler_recipe</t>
-        </is>
-      </c>
-      <c r="B74" s="3" t="inlineStr">
-        <is>
-          <t>Bouclier de gel</t>
-        </is>
-      </c>
-      <c r="C74" s="3" t="inlineStr">
-        <is>
-          <t>slime_buckler</t>
-        </is>
-      </c>
-      <c r="D74" s="3" t="inlineStr">
-        <is>
-          <t>shield</t>
-        </is>
-      </c>
-      <c r="E74" s="3" t="inlineStr">
-        <is>
-          <t>main_droite</t>
-        </is>
-      </c>
-      <c r="F74" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G74" s="4" t="inlineStr">
         <is>
           <t>slime_gel ×3
 wood_log ×2
@@ -6097,36 +6060,36 @@
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" t="inlineStr">
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
         <is>
           <t>slime_greatblade_recipe</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B74" s="3" t="inlineStr">
         <is>
           <t>Lame visqueuse colossale</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C74" s="3" t="inlineStr">
         <is>
           <t>slime_greatblade</t>
         </is>
       </c>
-      <c r="D75" t="inlineStr">
+      <c r="D74" s="3" t="inlineStr">
         <is>
           <t>weapon</t>
         </is>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E74" s="3" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F75" t="n">
-        <v>1</v>
-      </c>
-      <c r="G75" s="5" t="inlineStr">
+      <c r="F74" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G74" s="4" t="inlineStr">
         <is>
           <t>slime_gel ×9
 wood_log ×6
@@ -6134,36 +6097,36 @@
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="3" t="inlineStr">
+    <row r="75">
+      <c r="A75" t="inlineStr">
         <is>
           <t>slime_tower_shield_recipe</t>
         </is>
       </c>
-      <c r="B76" s="3" t="inlineStr">
+      <c r="B75" t="inlineStr">
         <is>
           <t>Tour de gel</t>
         </is>
       </c>
-      <c r="C76" s="3" t="inlineStr">
+      <c r="C75" t="inlineStr">
         <is>
           <t>slime_tower_shield</t>
         </is>
       </c>
-      <c r="D76" s="3" t="inlineStr">
+      <c r="D75" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E76" s="3" t="inlineStr">
+      <c r="E75" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F76" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G76" s="4" t="inlineStr">
+      <c r="F75" t="n">
+        <v>1</v>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
         <is>
           <t>slime_gel ×12
 wood_log ×9
@@ -6171,36 +6134,36 @@
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>gobelin_buckler_recipe</t>
         </is>
       </c>
-      <c r="B77" t="inlineStr">
+      <c r="B76" s="3" t="inlineStr">
         <is>
           <t>Rondache gobeline</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
+      <c r="C76" s="3" t="inlineStr">
         <is>
           <t>gobelin_buckler</t>
         </is>
       </c>
-      <c r="D77" t="inlineStr">
+      <c r="D76" s="3" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E77" t="inlineStr">
+      <c r="E76" s="3" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F77" t="n">
-        <v>1</v>
-      </c>
-      <c r="G77" s="5" t="inlineStr">
+      <c r="F76" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G76" s="4" t="inlineStr">
         <is>
           <t>gobelin_tooth ×3
 iron_ingot ×1
@@ -6208,36 +6171,36 @@
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="3" t="inlineStr">
+    <row r="77">
+      <c r="A77" t="inlineStr">
         <is>
           <t>gobelin_greataxe_recipe</t>
         </is>
       </c>
-      <c r="B78" s="3" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>Grande hache gobeline</t>
         </is>
       </c>
-      <c r="C78" s="3" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>gobelin_greataxe</t>
         </is>
       </c>
-      <c r="D78" s="3" t="inlineStr">
+      <c r="D77" t="inlineStr">
         <is>
           <t>weapon</t>
         </is>
       </c>
-      <c r="E78" s="3" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F78" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G78" s="4" t="inlineStr">
+      <c r="F77" t="n">
+        <v>1</v>
+      </c>
+      <c r="G77" s="5" t="inlineStr">
         <is>
           <t>gobelin_tooth ×12
 iron_ingot ×6
@@ -6245,36 +6208,36 @@
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
         <is>
           <t>gobelin_warshield_recipe</t>
         </is>
       </c>
-      <c r="B79" t="inlineStr">
+      <c r="B78" s="3" t="inlineStr">
         <is>
           <t>Pavois gobelin</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr">
+      <c r="C78" s="3" t="inlineStr">
         <is>
           <t>gobelin_warshield</t>
         </is>
       </c>
-      <c r="D79" t="inlineStr">
+      <c r="D78" s="3" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr">
+      <c r="E78" s="3" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F79" t="n">
-        <v>1</v>
-      </c>
-      <c r="G79" s="5" t="inlineStr">
+      <c r="F78" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="4" t="inlineStr">
         <is>
           <t>gobelin_tooth ×9
 iron_ingot ×3
@@ -6283,36 +6246,36 @@
         </is>
       </c>
     </row>
-    <row r="80">
-      <c r="A80" s="3" t="inlineStr">
+    <row r="79">
+      <c r="A79" t="inlineStr">
         <is>
           <t>leather_dagger_recipe</t>
         </is>
       </c>
-      <c r="B80" s="3" t="inlineStr">
+      <c r="B79" t="inlineStr">
         <is>
           <t>Dague en cuir</t>
         </is>
       </c>
-      <c r="C80" s="3" t="inlineStr">
+      <c r="C79" t="inlineStr">
         <is>
           <t>leather_dagger</t>
         </is>
       </c>
-      <c r="D80" s="3" t="inlineStr">
+      <c r="D79" t="inlineStr">
         <is>
           <t>weapon</t>
         </is>
       </c>
-      <c r="E80" s="3" t="inlineStr">
+      <c r="E79" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F80" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G80" s="4" t="inlineStr">
+      <c r="F79" t="n">
+        <v>1</v>
+      </c>
+      <c r="G79" s="5" t="inlineStr">
         <is>
           <t>leather_strip ×2
 wood_log ×2
@@ -6320,36 +6283,36 @@
         </is>
       </c>
     </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="3" t="inlineStr">
         <is>
           <t>leather_buckler_recipe</t>
         </is>
       </c>
-      <c r="B81" t="inlineStr">
+      <c r="B80" s="3" t="inlineStr">
         <is>
           <t>Rondache en cuir</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
+      <c r="C80" s="3" t="inlineStr">
         <is>
           <t>leather_buckler</t>
         </is>
       </c>
-      <c r="D81" t="inlineStr">
+      <c r="D80" s="3" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E81" t="inlineStr">
+      <c r="E80" s="3" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F81" t="n">
-        <v>1</v>
-      </c>
-      <c r="G81" s="5" t="inlineStr">
+      <c r="F80" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G80" s="4" t="inlineStr">
         <is>
           <t>leather_strip ×2
 wood_log ×2
@@ -6357,36 +6320,36 @@
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
+    <row r="81">
+      <c r="A81" t="inlineStr">
         <is>
           <t>leather_greatsword_recipe</t>
         </is>
       </c>
-      <c r="B82" s="3" t="inlineStr">
+      <c r="B81" t="inlineStr">
         <is>
           <t>Grande lame en cuir</t>
         </is>
       </c>
-      <c r="C82" s="3" t="inlineStr">
+      <c r="C81" t="inlineStr">
         <is>
           <t>leather_greatsword</t>
         </is>
       </c>
-      <c r="D82" s="3" t="inlineStr">
+      <c r="D81" t="inlineStr">
         <is>
           <t>weapon</t>
         </is>
       </c>
-      <c r="E82" s="3" t="inlineStr">
+      <c r="E81" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F82" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G82" s="4" t="inlineStr">
+      <c r="F81" t="n">
+        <v>1</v>
+      </c>
+      <c r="G81" s="5" t="inlineStr">
         <is>
           <t>leather_strip ×9
 wood_log ×6
@@ -6394,36 +6357,36 @@
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" t="inlineStr">
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
         <is>
           <t>leather_tower_shield_recipe</t>
         </is>
       </c>
-      <c r="B83" t="inlineStr">
+      <c r="B82" s="3" t="inlineStr">
         <is>
           <t>Tour en cuir</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
+      <c r="C82" s="3" t="inlineStr">
         <is>
           <t>leather_tower_shield</t>
         </is>
       </c>
-      <c r="D83" t="inlineStr">
+      <c r="D82" s="3" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr">
+      <c r="E82" s="3" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F83" t="n">
-        <v>1</v>
-      </c>
-      <c r="G83" s="5" t="inlineStr">
+      <c r="F82" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G82" s="4" t="inlineStr">
         <is>
           <t>leather_strip ×9
 wood_log ×9
@@ -6431,36 +6394,36 @@
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="3" t="inlineStr">
+    <row r="83">
+      <c r="A83" t="inlineStr">
         <is>
           <t>linen_rapier_recipe</t>
         </is>
       </c>
-      <c r="B84" s="3" t="inlineStr">
+      <c r="B83" t="inlineStr">
         <is>
           <t>Rapière en lin</t>
         </is>
       </c>
-      <c r="C84" s="3" t="inlineStr">
+      <c r="C83" t="inlineStr">
         <is>
           <t>linen_rapier</t>
         </is>
       </c>
-      <c r="D84" s="3" t="inlineStr">
+      <c r="D83" t="inlineStr">
         <is>
           <t>weapon</t>
         </is>
       </c>
-      <c r="E84" s="3" t="inlineStr">
+      <c r="E83" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F84" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G84" s="4" t="inlineStr">
+      <c r="F83" t="n">
+        <v>1</v>
+      </c>
+      <c r="G83" s="5" t="inlineStr">
         <is>
           <t>linen_cloth ×2
 wood_log ×2
@@ -6468,36 +6431,36 @@
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
         <is>
           <t>linen_aegis_recipe</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B84" s="3" t="inlineStr">
         <is>
           <t>Égide en lin</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C84" s="3" t="inlineStr">
         <is>
           <t>linen_aegis</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D84" s="3" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E84" s="3" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F85" t="n">
-        <v>1</v>
-      </c>
-      <c r="G85" s="5" t="inlineStr">
+      <c r="F84" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G84" s="4" t="inlineStr">
         <is>
           <t>linen_cloth ×2
 wood_log ×2
@@ -6505,36 +6468,36 @@
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" s="3" t="inlineStr">
+    <row r="85">
+      <c r="A85" t="inlineStr">
         <is>
           <t>linen_greatblade_recipe</t>
         </is>
       </c>
-      <c r="B86" s="3" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>Grande lame en lin</t>
         </is>
       </c>
-      <c r="C86" s="3" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>linen_greatblade</t>
         </is>
       </c>
-      <c r="D86" s="3" t="inlineStr">
+      <c r="D85" t="inlineStr">
         <is>
           <t>weapon</t>
         </is>
       </c>
-      <c r="E86" s="3" t="inlineStr">
+      <c r="E85" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F86" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G86" s="4" t="inlineStr">
+      <c r="F85" t="n">
+        <v>1</v>
+      </c>
+      <c r="G85" s="5" t="inlineStr">
         <is>
           <t>linen_cloth ×9
 wood_log ×6
@@ -6542,36 +6505,36 @@
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="3" t="inlineStr">
         <is>
           <t>linen_tower_shield_recipe</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B86" s="3" t="inlineStr">
         <is>
           <t>Tour en lin</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C86" s="3" t="inlineStr">
         <is>
           <t>linen_tower_shield</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D86" s="3" t="inlineStr">
         <is>
           <t>shield</t>
         </is>
       </c>
-      <c r="E87" t="inlineStr">
+      <c r="E86" s="3" t="inlineStr">
         <is>
           <t>main_droite</t>
         </is>
       </c>
-      <c r="F87" t="n">
-        <v>1</v>
-      </c>
-      <c r="G87" s="5" t="inlineStr">
+      <c r="F86" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G86" s="4" t="inlineStr">
         <is>
           <t>linen_cloth ×9
 wood_log ×9
@@ -10361,10 +10324,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P19"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
@@ -10715,17 +10678,17 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>two_handed_iron_sword</t>
+          <t>iron_dagger</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Espadon de fer</t>
+          <t>Dague en fer</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>common</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -10735,11 +10698,11 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>10</v>
+        <v>3</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -10748,46 +10711,46 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>35</v>
+        <v>12</v>
       </c>
       <c r="O6" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>Une longue lame qui demande de tenir des deux mains.</t>
+          <t>Dague affûtée, légère et discrète.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>iron_dagger</t>
+          <t>goblin_blade</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Dague en fer</t>
+          <t>Lame gobeline</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>uncommon</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -10801,7 +10764,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -10810,46 +10773,46 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="O7" t="n">
         <v>0</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>Dague affûtée, légère et discrète.</t>
+          <t>Lame ébréchée mais redoutable, taillée d'os de gobelin.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>goblin_blade</t>
+          <t>leather_main_droite</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Lame gobeline</t>
+          <t>Lame en cuir</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>uncommon</t>
+          <t>common</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -10863,10 +10826,10 @@
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>0</v>
@@ -10875,10 +10838,10 @@
         <v>0</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="K8" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L8" s="3" t="n">
         <v>0</v>
@@ -10887,26 +10850,26 @@
         <v>0</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>22</v>
+        <v>4</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>Lame ébréchée mais redoutable, taillée d'os de gobelin.</t>
+          <t>Pièce de la panoplie leather — bonus de set actif dès 2 pièces.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>leather_main_droite</t>
+          <t>linen_main_droite</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Lame en cuir</t>
+          <t>Lame en lin</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -10928,7 +10891,7 @@
         <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H9" t="n">
         <v>0</v>
@@ -10937,7 +10900,7 @@
         <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K9" t="n">
         <v>1</v>
@@ -10956,19 +10919,19 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>Pièce de la panoplie leather — bonus de set actif dès 2 pièces.</t>
+          <t>Pièce de la panoplie linen — bonus de set actif dès 2 pièces.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>linen_main_droite</t>
+          <t>iron_sword</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Lame en lin</t>
+          <t>Épée en fer</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -10987,22 +10950,22 @@
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>0</v>
       </c>
       <c r="J10" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K10" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L10" s="3" t="n">
         <v>0</v>
@@ -11011,31 +10974,31 @@
         <v>0</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
-          <t>Pièce de la panoplie linen — bonus de set actif dès 2 pièces.</t>
+          <t>Variante équilibrée de la dague en fer — atk + un peu de def/PV.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>iron_sword</t>
+          <t>iron_greatsword</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Épée en fer</t>
+          <t>Espadon en fer</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -11045,59 +11008,59 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>-5</v>
       </c>
       <c r="H11" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="J11" t="n">
         <v>0</v>
       </c>
       <c r="K11" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="L11" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>18</v>
+        <v>60</v>
       </c>
       <c r="O11" t="n">
         <v>0</v>
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>Variante équilibrée de la dague en fer — atk + un peu de def/PV.</t>
+          <t>Lame à 2 mains — frappe lourde mais on s'expose en attaquant.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>iron_greatsword</t>
+          <t>slime_morningstar</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Espadon en fer</t>
+          <t>Morningstar visqueuse</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>common</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -11107,59 +11070,59 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>-5</v>
+        <v>0</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="J12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="K12" s="3" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="L12" s="3" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M12" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>60</v>
+        <v>22</v>
       </c>
       <c r="O12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P12" s="3" t="inlineStr">
         <is>
-          <t>Lame à 2 mains — frappe lourde mais on s'expose en attaquant.</t>
+          <t>Variante régen de la lame visqueuse — atk soutenue + un peu de régen.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>slime_morningstar</t>
+          <t>slime_greatblade</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Morningstar visqueuse</t>
+          <t>Lame visqueuse colossale</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -11169,17 +11132,17 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>-4</v>
       </c>
       <c r="H13" t="n">
-        <v>0</v>
+        <v>-6</v>
       </c>
       <c r="I13" t="n">
         <v>0</v>
@@ -11194,29 +11157,29 @@
         <v>0</v>
       </c>
       <c r="M13" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="O13" t="n">
         <v>0</v>
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>Variante régen de la lame visqueuse — atk soutenue + un peu de régen.</t>
+          <t>2 mains — frappe massive, on perd en résilience.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>slime_greatblade</t>
+          <t>gobelin_greataxe</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Lame visqueuse colossale</t>
+          <t>Grande hache gobeline</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -11235,20 +11198,20 @@
         </is>
       </c>
       <c r="F14" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="G14" s="3" t="n">
+        <v>-2</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>-2</v>
+      </c>
+      <c r="J14" s="3" t="n">
         <v>15</v>
       </c>
-      <c r="G14" s="3" t="n">
-        <v>-4</v>
-      </c>
-      <c r="H14" s="3" t="n">
-        <v>-6</v>
-      </c>
-      <c r="I14" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="3" t="n">
-        <v>0</v>
-      </c>
       <c r="K14" s="3" t="n">
         <v>0</v>
       </c>
@@ -11259,31 +11222,31 @@
         <v>0</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>70</v>
+        <v>80</v>
       </c>
       <c r="O14" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P14" s="3" t="inlineStr">
         <is>
-          <t>2 mains — frappe massive, on perd en résilience.</t>
+          <t>2 mains — crit massifs, on se découvre complètement.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>gobelin_greataxe</t>
+          <t>leather_dagger</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Grande hache gobeline</t>
+          <t>Dague en cuir</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>common</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -11293,26 +11256,26 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>18</v>
+        <v>2</v>
       </c>
       <c r="G15" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
       </c>
       <c r="I15" t="n">
-        <v>-2</v>
+        <v>0</v>
       </c>
       <c r="J15" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="L15" t="n">
         <v>0</v>
@@ -11321,31 +11284,31 @@
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>80</v>
+        <v>14</v>
       </c>
       <c r="O15" t="n">
         <v>0</v>
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2 mains — crit massifs, on se découvre complètement.</t>
+          <t>Variante offensive de la lame en cuir — un peu d'attaque en plus.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>leather_dagger</t>
+          <t>leather_greatsword</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Dague en cuir</t>
+          <t>Grande lame en cuir</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -11355,27 +11318,27 @@
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="F16" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="G16" s="3" t="n">
+        <v>-1</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="G16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K16" s="3" t="n">
-        <v>1</v>
-      </c>
       <c r="L16" s="3" t="n">
         <v>0</v>
       </c>
@@ -11383,31 +11346,31 @@
         <v>0</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="O16" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P16" s="3" t="inlineStr">
         <is>
-          <t>Variante offensive de la lame en cuir — un peu d'attaque en plus.</t>
+          <t>2 mains — atk solide pour la panoplie cuir, on perd en couverture.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>leather_greatsword</t>
+          <t>linen_rapier</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Grande lame en cuir</t>
+          <t>Rapière en lin</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>rare</t>
+          <t>common</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -11417,59 +11380,59 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>oui</t>
+          <t>non</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="G17" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
       </c>
       <c r="I17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J17" t="n">
         <v>0</v>
       </c>
       <c r="K17" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="L17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>50</v>
+        <v>16</v>
       </c>
       <c r="O17" t="n">
         <v>0</v>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2 mains — atk solide pour la panoplie cuir, on perd en couverture.</t>
+          <t>Variante speed/crit de la lame en lin — précise mais fragile.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>linen_rapier</t>
+          <t>linen_greatblade</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Rapière en lin</t>
+          <t>Grande lame en lin</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>common</t>
+          <t>rare</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -11479,102 +11442,40 @@
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>oui</t>
         </is>
       </c>
       <c r="F18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>0</v>
+        <v>-3</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J18" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="K18" s="3" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="L18" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>16</v>
+        <v>55</v>
       </c>
       <c r="O18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="P18" s="3" t="inlineStr">
-        <is>
-          <t>Variante speed/crit de la lame en lin — précise mais fragile.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>linen_greatblade</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Grande lame en lin</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>rare</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>main_droite</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-      <c r="F19" t="n">
-        <v>0</v>
-      </c>
-      <c r="G19" t="n">
-        <v>-3</v>
-      </c>
-      <c r="H19" t="n">
-        <v>0</v>
-      </c>
-      <c r="I19" t="n">
-        <v>3</v>
-      </c>
-      <c r="J19" t="n">
-        <v>6</v>
-      </c>
-      <c r="K19" t="n">
-        <v>-1</v>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
-      </c>
-      <c r="M19" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" t="n">
-        <v>55</v>
-      </c>
-      <c r="O19" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" t="inlineStr">
         <is>
           <t>2 mains — crit dmg massif mais peu de couverture.</t>
         </is>

</xml_diff>

<commit_message>
Migre 6 boucliers main_gauche → main_droite (slot canonique unique)
Avec la convention V2 (un item main peut s'équiper indifféremment dans
n'importe quelle main), tous les hand items doivent avoir leur slot
canonique = main_droite. 6 anciens boucliers conservaient un slot
canonique main_gauche, ce qui n'était plus cohérent et faussait le
groupage par slot dans /panoplie (les boucliers étaient affichés
séparément des armes/2-mains dans une rubrique main_gauche).

Items migrés :
- wooden_shield, iron_buckler, slime_shield
- leather_main_gauche, gobelin_main_gauche, linen_main_gauche

Audit complet effectué : pas de doublons de noms, pas d'items inaccessibles,
pas de recettes/shop/drops orphelins, références sets/mobs/titres/skill
tree toutes valides.

Régénère sakura_content.xlsx.
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 2026-05-07 19:19 UTC</t>
+          <t>Généré le 2026-05-07 19:24 UTC</t>
         </is>
       </c>
     </row>
@@ -3791,7 +3791,7 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="F11" t="n">
@@ -3827,7 +3827,7 @@
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="F12" s="3" t="n">
@@ -4588,7 +4588,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="F33" t="n">
@@ -4736,7 +4736,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="F37" t="n">
@@ -5103,7 +5103,7 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="F47" t="n">
@@ -5394,7 +5394,7 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="F55" t="n">
@@ -11613,7 +11613,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr">
@@ -11675,7 +11675,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -11737,7 +11737,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -11799,7 +11799,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -11861,7 +11861,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -11923,7 +11923,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>main_gauche</t>
+          <t>main_droite</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">

</xml_diff>

<commit_message>
Refonte /shop : achat uniquement, sans drops de mob, UI soignée
Conceptuel :
- Suppression totale de la VENTE joueur→shop : commande /sell retirée,
  embed de vente retiré. On ne peut plus QUE acheter.
- Les drops de mob (slime_gel, gobelin_tooth) ne sont plus en boutique —
  ils servent uniquement au craft. Retirés de shop_items.json + DB.

Esthétique (shop_view) :
- Onglets par catégorie (inchangé), mais items présentés proprement :
  icône de catégorie + pastille de rareté (⚪🟢🔵🟣🟠) + description +
  prix d'achat + raccourci /buy. Tri par prix croissant. Footer clair
  "La revente n'existe pas". Plus de lignes vente/stock/saturation.

shop_cog allégé (plus de /sell, autocomplete, imports vente). Les services
de vente (SellToShopUseCase, ShopPricingService.current_sell_price)
subsistent car encore utilisés côté admin, mais plus côté joueur.

Docs (CLAUDE.md + tuto.txt) + xlsx à jour. 383 tests verts.
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 2026-05-25 19:37 UTC</t>
+          <t>Généré le 2026-05-25 19:53 UTC</t>
         </is>
       </c>
     </row>
@@ -6553,7 +6553,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -6781,30 +6781,30 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>slime_gel</t>
+          <t>potion_soin_i</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gelée de Slime</t>
+          <t>Potion de soin I</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>resource</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>30</v>
       </c>
       <c r="E7" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -6815,30 +6815,30 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>gobelin_tooth</t>
+          <t>potion_soin_ii</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Dent de Gobelin</t>
+          <t>Potion de soin II</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>resource</t>
+          <t>consumable</t>
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>4</v>
+        <v>70</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>100</v>
+        <v>30</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
@@ -6849,12 +6849,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>potion_soin_i</t>
+          <t>potion_soin_iii</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Potion de soin I</t>
+          <t>Potion de soin III</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -6863,86 +6863,18 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>30</v>
+        <v>150</v>
       </c>
       <c r="E9" t="n">
-        <v>8</v>
+        <v>40</v>
       </c>
       <c r="F9" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="G9" t="n">
-        <v>50</v>
+        <v>20</v>
       </c>
       <c r="H9" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t>potion_soin_ii</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>Potion de soin II</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="D10" s="3" t="n">
-        <v>70</v>
-      </c>
-      <c r="E10" s="3" t="n">
-        <v>18</v>
-      </c>
-      <c r="F10" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="G10" s="3" t="n">
-        <v>30</v>
-      </c>
-      <c r="H10" s="3" t="inlineStr">
-        <is>
-          <t>oui</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>potion_soin_iii</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Potion de soin III</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>consumable</t>
-        </is>
-      </c>
-      <c r="D11" t="n">
-        <v>150</v>
-      </c>
-      <c r="E11" t="n">
-        <v>40</v>
-      </c>
-      <c r="F11" t="n">
-        <v>15</v>
-      </c>
-      <c r="G11" t="n">
-        <v>20</v>
-      </c>
-      <c r="H11" t="inlineStr">
         <is>
           <t>oui</t>
         </is>

</xml_diff>

<commit_message>
Gobelin Assassin : passé à ~2K de puissance (palier C, PV564/ATK53/DEF31, score 2025=2K)
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 2026-05-25 22:09 UTC</t>
+          <t>Généré le 2026-05-25 22:18 UTC</t>
         </is>
       </c>
     </row>
@@ -9476,12 +9476,12 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>gobelin_assassin</t>
+          <t>gobelin_ballon</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Gobelin Assassin</t>
+          <t>Gobelin Ballon</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -9490,71 +9490,67 @@
         </is>
       </c>
       <c r="D6" s="3" t="n">
-        <v>286</v>
+        <v>557</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>28</v>
+        <v>36</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="H6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>100</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>175</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>84</v>
+      </c>
+      <c r="N6" s="3" t="n">
         <v>20</v>
       </c>
-      <c r="I6" s="3" t="n">
-        <v>150</v>
-      </c>
-      <c r="J6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="K6" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="3" t="n">
-        <v>144</v>
-      </c>
-      <c r="M6" s="3" t="n">
-        <v>69</v>
-      </c>
-      <c r="N6" s="3" t="n">
-        <v>10</v>
-      </c>
       <c r="O6" s="3" t="n">
-        <v>548</v>
+        <v>1018</v>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>F+</t>
-        </is>
-      </c>
-      <c r="Q6" s="3" t="inlineStr">
-        <is>
-          <t>sang_gobelin_hq ×1-1 (15%)</t>
-        </is>
-      </c>
+          <t>E-</t>
+        </is>
+      </c>
+      <c r="Q6" s="3" t="inlineStr"/>
       <c r="R6" s="3" t="inlineStr">
         <is>
-          <t>gobelin_assassin.png</t>
+          <t>gobelin_ballon.png</t>
         </is>
       </c>
       <c r="S6" s="3" t="inlineStr">
         <is>
-          <t>Une créature discrète.</t>
+          <t>Un groupe de créatures inventives.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>gobelin_ballon</t>
+          <t>gobelin_geant</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Gobelin Ballon</t>
+          <t>Gobelin Géant</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -9563,13 +9559,13 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>557</v>
+        <v>955</v>
       </c>
       <c r="E7" t="n">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="F7" t="n">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="G7" t="n">
         <v>5</v>
@@ -9587,43 +9583,43 @@
         <v>0</v>
       </c>
       <c r="L7" t="n">
-        <v>175</v>
+        <v>206</v>
       </c>
       <c r="M7" t="n">
-        <v>84</v>
+        <v>99</v>
       </c>
       <c r="N7" t="n">
         <v>20</v>
       </c>
       <c r="O7" t="n">
-        <v>1018</v>
+        <v>1221</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>E-</t>
+          <t>E</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr">
         <is>
-          <t>gobelin_ballon.png</t>
+          <t>gobelin_geant.png</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Un groupe de créatures inventives.</t>
+          <t>Une créature imposante.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>gobelin_geant</t>
+          <t>gobelin_runique</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Gobelin Géant</t>
+          <t>Gobelin Runique</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
@@ -9632,13 +9628,13 @@
         </is>
       </c>
       <c r="D8" s="3" t="n">
-        <v>955</v>
+        <v>573</v>
       </c>
       <c r="E8" s="3" t="n">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>5</v>
@@ -9656,43 +9652,43 @@
         <v>0</v>
       </c>
       <c r="L8" s="3" t="n">
-        <v>206</v>
+        <v>238</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>99</v>
+        <v>114</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>20</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>1221</v>
+        <v>1611</v>
       </c>
       <c r="P8" s="3" t="inlineStr">
         <is>
-          <t>E</t>
+          <t>E+</t>
         </is>
       </c>
       <c r="Q8" s="3" t="inlineStr"/>
       <c r="R8" s="3" t="inlineStr">
         <is>
-          <t>gobelin_geant.png</t>
+          <t>gobelin_runique.png</t>
         </is>
       </c>
       <c r="S8" s="3" t="inlineStr">
         <is>
-          <t>Une créature imposante.</t>
+          <t>Une créature mystérieuse.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>gobelin_runique</t>
+          <t>gobelin_superieur</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Gobelin Runique</t>
+          <t>Gobelin Supérieur</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -9701,13 +9697,13 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>573</v>
+        <v>876</v>
       </c>
       <c r="E9" t="n">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="F9" t="n">
-        <v>15</v>
+        <v>36</v>
       </c>
       <c r="G9" t="n">
         <v>5</v>
@@ -9725,43 +9721,47 @@
         <v>0</v>
       </c>
       <c r="L9" t="n">
-        <v>238</v>
+        <v>300</v>
       </c>
       <c r="M9" t="n">
-        <v>114</v>
+        <v>144</v>
       </c>
       <c r="N9" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="O9" t="n">
-        <v>1611</v>
+        <v>2442</v>
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>E+</t>
-        </is>
-      </c>
-      <c r="Q9" t="inlineStr"/>
+          <t>D-</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>sang_gobelin_hq ×1-1 (15%)</t>
+        </is>
+      </c>
       <c r="R9" t="inlineStr">
         <is>
-          <t>gobelin_runique.png</t>
+          <t>gobelin_superieur.png</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Une créature mystérieuse.</t>
+          <t>Une créature supérieure.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>gobelin_superieur</t>
+          <t>gobelin_assassin</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Gobelin Supérieur</t>
+          <t>Gobelin Assassin</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -9770,22 +9770,22 @@
         </is>
       </c>
       <c r="D10" s="3" t="n">
-        <v>876</v>
+        <v>564</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>100</v>
+        <v>150</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>0</v>
@@ -9794,16 +9794,16 @@
         <v>0</v>
       </c>
       <c r="L10" s="3" t="n">
-        <v>300</v>
+        <v>325</v>
       </c>
       <c r="M10" s="3" t="n">
-        <v>144</v>
+        <v>156</v>
       </c>
       <c r="N10" s="3" t="n">
         <v>10</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>2442</v>
+        <v>2025</v>
       </c>
       <c r="P10" s="3" t="inlineStr">
         <is>
@@ -9817,12 +9817,12 @@
       </c>
       <c r="R10" s="3" t="inlineStr">
         <is>
-          <t>gobelin_superieur.png</t>
+          <t>gobelin_assassin.png</t>
         </is>
       </c>
       <c r="S10" s="3" t="inlineStr">
         <is>
-          <t>Une créature supérieure.</t>
+          <t>Une créature discrète.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Équilibrage panoplies : remonte un peu la puissance (set ~5× base)
TARGET_POWER 230 → 290, cœurs arme/bouclier (atk 6→8, def 5→7) et
bonus de set relevés. Autotune garde les familles équilibrées (~277-304).

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 2026-05-26 00:11 UTC</t>
+          <t>Généré le 2026-05-26 00:32 UTC</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -908,7 +908,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -970,7 +970,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -985,7 +985,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" t="n">
         <v>6</v>
@@ -1156,7 +1156,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -1171,7 +1171,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -1332,7 +1332,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -1518,7 +1518,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1580,7 +1580,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>0</v>
@@ -1766,7 +1766,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1942,7 +1942,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -2066,7 +2066,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -2081,7 +2081,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>6</v>
@@ -2314,7 +2314,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -2329,7 +2329,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -2614,7 +2614,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -2676,7 +2676,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -2862,7 +2862,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -3100,7 +3100,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -3162,7 +3162,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -3224,7 +3224,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -3239,7 +3239,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N5" t="n">
         <v>6</v>
@@ -3472,7 +3472,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -3487,7 +3487,7 @@
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="N9" t="n">
         <v>12</v>
@@ -17318,7 +17318,7 @@
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="25" customWidth="1" min="7" max="7"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
     <col width="26" customWidth="1" min="9" max="9"/>
   </cols>
@@ -17401,17 +17401,17 @@
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>defense_flat +2</t>
+          <t>defense_flat +3</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
         <is>
-          <t>defense_flat +3</t>
+          <t>defense_flat +5</t>
         </is>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>defense_flat +4</t>
+          <t>defense_flat +7</t>
         </is>
       </c>
     </row>
@@ -17451,12 +17451,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>dodge_flat +3</t>
+          <t>dodge_flat +4</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>dodge_flat +4</t>
+          <t>dodge_flat +6</t>
         </is>
       </c>
     </row>
@@ -17486,22 +17486,22 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>hp_regeneration_flat +3</t>
+          <t>hp_regeneration_flat +4</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>hp_regeneration_flat +6</t>
+          <t>hp_regeneration_flat +8</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
-          <t>hp_regeneration_flat +10</t>
+          <t>hp_regeneration_flat +13</t>
         </is>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>hp_regeneration_flat +15</t>
+          <t>hp_regeneration_flat +18</t>
         </is>
       </c>
     </row>
@@ -17536,17 +17536,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>crit_chance_flat +1</t>
+          <t>crit_chance_flat +2</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>crit_chance_flat +2</t>
+          <t>crit_chance_flat +3</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>crit_chance_flat +3</t>
+          <t>crit_chance_flat +4</t>
         </is>
       </c>
     </row>
@@ -17576,22 +17576,22 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>crit_damage_flat +2</t>
+          <t>crit_damage_flat +3</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>crit_damage_flat +4</t>
+          <t>crit_damage_flat +6</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>crit_damage_flat +6</t>
+          <t>crit_damage_flat +9</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>crit_damage_flat +10</t>
+          <t>crit_damage_flat +14</t>
         </is>
       </c>
     </row>
@@ -17626,17 +17626,17 @@
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>crit_chance_flat +2</t>
+          <t>crit_chance_flat +3</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>crit_chance_flat +3</t>
+          <t>crit_chance_flat +5</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>crit_chance_flat +5</t>
+          <t>crit_chance_flat +6</t>
         </is>
       </c>
     </row>
@@ -17666,22 +17666,22 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>hp_regeneration_flat +5</t>
+          <t>hp_regeneration_flat +6</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>hp_regeneration_flat +9</t>
+          <t>hp_regeneration_flat +12</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>hp_regeneration_flat +14</t>
+          <t>hp_regeneration_flat +19</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>hp_regeneration_flat +21</t>
+          <t>hp_regeneration_flat +26</t>
         </is>
       </c>
     </row>
@@ -18222,7 +18222,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -18346,7 +18346,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -18408,7 +18408,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>1</v>
@@ -18470,7 +18470,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -18532,7 +18532,7 @@
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>0</v>
@@ -18594,7 +18594,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G9" t="n">
         <v>0</v>
@@ -18656,7 +18656,7 @@
         </is>
       </c>
       <c r="F10" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>1</v>
@@ -18718,7 +18718,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G11" t="n">
         <v>2</v>
@@ -18780,7 +18780,7 @@
         </is>
       </c>
       <c r="F12" s="3" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>0</v>
@@ -18842,7 +18842,7 @@
         </is>
       </c>
       <c r="F13" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G13" t="n">
         <v>-3</v>
@@ -18904,7 +18904,7 @@
         </is>
       </c>
       <c r="F14" s="3" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>0</v>
@@ -18966,7 +18966,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G15" t="n">
         <v>0</v>
@@ -19028,7 +19028,7 @@
         </is>
       </c>
       <c r="F16" s="3" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>-2</v>
@@ -19090,7 +19090,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G17" t="n">
         <v>0</v>
@@ -19152,7 +19152,7 @@
         </is>
       </c>
       <c r="F18" s="3" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>-3</v>
@@ -19214,7 +19214,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G19" t="n">
         <v>0</v>
@@ -19276,7 +19276,7 @@
         </is>
       </c>
       <c r="F20" s="3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G20" s="3" t="n">
         <v>0</v>
@@ -19338,7 +19338,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G21" t="n">
         <v>0</v>
@@ -19400,7 +19400,7 @@
         </is>
       </c>
       <c r="F22" s="3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G22" s="3" t="n">
         <v>0</v>
@@ -19462,7 +19462,7 @@
         </is>
       </c>
       <c r="F23" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="G23" t="n">
         <v>0</v>
@@ -19524,7 +19524,7 @@
         </is>
       </c>
       <c r="F24" s="3" t="n">
-        <v>18</v>
+        <v>24</v>
       </c>
       <c r="G24" s="3" t="n">
         <v>-3</v>
@@ -19765,7 +19765,7 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H3" t="n">
         <v>4</v>
@@ -19827,7 +19827,7 @@
         <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H4" s="3" t="n">
         <v>6</v>
@@ -19889,7 +19889,7 @@
         <v>0</v>
       </c>
       <c r="G5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H5" t="n">
         <v>0</v>
@@ -19951,7 +19951,7 @@
         <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H6" s="3" t="n">
         <v>0</v>
@@ -20013,7 +20013,7 @@
         <v>0</v>
       </c>
       <c r="G7" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H7" t="n">
         <v>0</v>
@@ -20075,7 +20075,7 @@
         <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H8" s="3" t="n">
         <v>4</v>
@@ -20137,7 +20137,7 @@
         <v>-4</v>
       </c>
       <c r="G9" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H9" t="n">
         <v>8</v>
@@ -20199,7 +20199,7 @@
         <v>0</v>
       </c>
       <c r="G10" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H10" s="3" t="n">
         <v>6</v>
@@ -20261,7 +20261,7 @@
         <v>-4</v>
       </c>
       <c r="G11" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H11" t="n">
         <v>12</v>
@@ -20323,7 +20323,7 @@
         <v>0</v>
       </c>
       <c r="G12" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H12" s="3" t="n">
         <v>0</v>
@@ -20385,7 +20385,7 @@
         <v>-4</v>
       </c>
       <c r="G13" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H13" t="n">
         <v>0</v>
@@ -20447,7 +20447,7 @@
         <v>0</v>
       </c>
       <c r="G14" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H14" s="3" t="n">
         <v>0</v>
@@ -20509,7 +20509,7 @@
         <v>-4</v>
       </c>
       <c r="G15" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H15" t="n">
         <v>0</v>
@@ -20571,7 +20571,7 @@
         <v>0</v>
       </c>
       <c r="G16" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="H16" s="3" t="n">
         <v>0</v>
@@ -20633,7 +20633,7 @@
         <v>-4</v>
       </c>
       <c r="G17" t="n">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="H17" t="n">
         <v>0</v>
@@ -20695,7 +20695,7 @@
         <v>0</v>
       </c>
       <c r="G18" s="3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H18" s="3" t="n">
         <v>0</v>
@@ -20757,7 +20757,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H19" t="n">
         <v>0</v>
@@ -20819,7 +20819,7 @@
         <v>-4</v>
       </c>
       <c r="G20" s="3" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H20" s="3" t="n">
         <v>0</v>
@@ -20881,7 +20881,7 @@
         <v>0</v>
       </c>
       <c r="G21" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H21" t="n">
         <v>9</v>
@@ -20943,7 +20943,7 @@
         <v>0</v>
       </c>
       <c r="G22" s="3" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="H22" s="3" t="n">
         <v>9</v>
@@ -21005,7 +21005,7 @@
         <v>-4</v>
       </c>
       <c r="G23" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="H23" t="n">
         <v>18</v>
@@ -21246,7 +21246,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -21432,7 +21432,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>0</v>
@@ -21556,7 +21556,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -21732,7 +21732,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -21791,10 +21791,10 @@
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -21918,7 +21918,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -22104,7 +22104,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -22342,7 +22342,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -22404,7 +22404,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -22652,7 +22652,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -22828,7 +22828,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -22890,7 +22890,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -22952,7 +22952,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -23200,7 +23200,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -23376,7 +23376,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -23500,7 +23500,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -23562,7 +23562,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -23748,7 +23748,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Panoplies : stats concentrées (chunky) au lieu d'éparpillées
Chaque pièce porte 1-2 stats nettes (+2/+3) plutôt qu'un +1 partout.
Distribution par rotation préservant les totaux par stat → power score
des familles inchangé (289-297). Fer en max_hp pur (sa def vit dans
bouclier+set), aucun slot d'armure vide.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 2026-05-26 00:32 UTC</t>
+          <t>Généré le 2026-05-26 00:43 UTC</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -793,7 +793,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0</v>
@@ -852,7 +852,7 @@
         <v>2</v>
       </c>
       <c r="J3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -970,7 +970,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -985,7 +985,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
         <v>6</v>
@@ -1038,7 +1038,7 @@
         <v>0</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -1100,7 +1100,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -1156,7 +1156,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>26</v>
+        <v>33</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -1171,7 +1171,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -1388,7 +1388,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -1397,10 +1397,10 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -1518,7 +1518,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1527,7 +1527,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -1580,7 +1580,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>0</v>
@@ -1595,7 +1595,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N6" s="3" t="n">
         <v>6</v>
@@ -1636,7 +1636,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -1648,7 +1648,7 @@
         <v>2</v>
       </c>
       <c r="J7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -1698,7 +1698,7 @@
         </is>
       </c>
       <c r="F8" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>0</v>
@@ -1707,10 +1707,10 @@
         <v>0</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>0</v>
@@ -1766,7 +1766,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1781,7 +1781,7 @@
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
         <v>12</v>
@@ -1942,7 +1942,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -1951,7 +1951,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0</v>
@@ -2066,7 +2066,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -2081,7 +2081,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>6</v>
@@ -2134,7 +2134,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -2196,7 +2196,7 @@
         <v>2</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -2258,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -2314,7 +2314,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -2329,7 +2329,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -2567,7 +2567,7 @@
         <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
         <v>14</v>
@@ -2676,7 +2676,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -2685,7 +2685,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -2732,7 +2732,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -2741,10 +2741,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -2794,7 +2794,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -2803,10 +2803,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -2862,7 +2862,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -2877,7 +2877,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>28</v>
@@ -3162,7 +3162,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -3171,7 +3171,7 @@
         <v>0</v>
       </c>
       <c r="K4" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L4" s="3" t="n">
         <v>0</v>
@@ -3224,7 +3224,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -3239,7 +3239,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
         <v>6</v>
@@ -3292,7 +3292,7 @@
         <v>0</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -3342,7 +3342,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -3351,10 +3351,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -3416,7 +3416,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>0</v>
@@ -3472,7 +3472,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>26</v>
+        <v>32</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -3487,7 +3487,7 @@
         <v>0</v>
       </c>
       <c r="M9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N9" t="n">
         <v>12</v>
@@ -21184,7 +21184,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -21193,7 +21193,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0</v>
@@ -21302,7 +21302,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
@@ -21311,10 +21311,10 @@
         <v>0</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>0</v>
@@ -21364,7 +21364,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -21376,7 +21376,7 @@
         <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -21432,7 +21432,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>0</v>
@@ -21447,7 +21447,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N6" s="3" t="n">
         <v>6</v>
@@ -21488,7 +21488,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -21497,10 +21497,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -21556,7 +21556,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -21571,7 +21571,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -21732,7 +21732,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -21741,7 +21741,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0</v>
@@ -21850,7 +21850,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
@@ -21859,10 +21859,10 @@
         <v>0</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>0</v>
@@ -21918,7 +21918,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -21933,7 +21933,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N5" t="n">
         <v>6</v>
@@ -21974,7 +21974,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -21983,10 +21983,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -22036,7 +22036,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -22045,10 +22045,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -22104,7 +22104,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -22119,7 +22119,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -22280,7 +22280,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -22289,7 +22289,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0</v>
@@ -22404,7 +22404,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -22419,7 +22419,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>6</v>
@@ -22460,7 +22460,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -22469,10 +22469,10 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -22522,7 +22522,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -22534,7 +22534,7 @@
         <v>2</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -22584,7 +22584,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -22593,10 +22593,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -22652,7 +22652,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -22667,7 +22667,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -22828,7 +22828,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -22837,7 +22837,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0</v>
@@ -22952,7 +22952,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -22967,7 +22967,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>6</v>
@@ -23008,7 +23008,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -23017,10 +23017,10 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -23132,7 +23132,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -23141,10 +23141,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -23200,7 +23200,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -23215,7 +23215,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -23376,7 +23376,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -23391,7 +23391,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N2" s="3" t="n">
         <v>10</v>
@@ -23432,7 +23432,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -23441,10 +23441,10 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -23500,7 +23500,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -23562,7 +23562,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -23571,7 +23571,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -23618,7 +23618,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -23630,7 +23630,7 @@
         <v>2</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -23680,7 +23680,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -23689,10 +23689,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -23748,7 +23748,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -23763,7 +23763,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>20</v>

</xml_diff>

<commit_message>
Panoplies : ~500 de bonus de puissance par set (chunk relevé à 6)
TARGET_POWER 290 → 560 (base ~58 → ~+500 de bonus). _CHUNK 2 → 6 pour
garder des stats concentrées (1-2 par pièce) malgré le budget plus gros.
Familles équilibrées (bonus 498-503). Vérif affiche désormais le bonus net.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/sakura_content.xlsx
+++ b/docs/sakura_content.xlsx
@@ -483,7 +483,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Généré le 2026-05-26 00:43 UTC</t>
+          <t>Généré le 2026-05-26 00:48 UTC</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -840,7 +840,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0</v>
+        <v>11</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -849,10 +849,10 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K3" t="n">
         <v>0</v>
@@ -908,7 +908,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>2</v>
+        <v>61</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -970,7 +970,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1038,7 +1038,7 @@
         <v>0</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -1100,7 +1100,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -1156,7 +1156,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -1332,7 +1332,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>2</v>
+        <v>61</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -1397,7 +1397,7 @@
         <v>0</v>
       </c>
       <c r="I3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J3" t="n">
         <v>0</v>
@@ -1518,7 +1518,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -1527,7 +1527,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -1580,7 +1580,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>0</v>
@@ -1645,10 +1645,10 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -1707,7 +1707,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J8" s="3" t="n">
         <v>0</v>
@@ -1766,7 +1766,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -1942,7 +1942,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>61</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -2066,7 +2066,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -2134,7 +2134,7 @@
         <v>0</v>
       </c>
       <c r="J5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -2193,10 +2193,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -2258,7 +2258,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -2314,7 +2314,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -2493,10 +2493,10 @@
         <v>0</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J2" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K2" s="3" t="n">
         <v>0</v>
@@ -2552,7 +2552,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -2614,7 +2614,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>2</v>
+        <v>61</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -2676,7 +2676,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -2741,7 +2741,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J6" s="3" t="n">
         <v>0</v>
@@ -2803,7 +2803,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -2862,7 +2862,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -3100,7 +3100,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>61</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -3162,7 +3162,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -3224,7 +3224,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>21</v>
+        <v>80</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -3292,7 +3292,7 @@
         <v>0</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -3342,7 +3342,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -3354,7 +3354,7 @@
         <v>0</v>
       </c>
       <c r="J7" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -3416,7 +3416,7 @@
         <v>0</v>
       </c>
       <c r="J8" s="3" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="K8" s="3" t="n">
         <v>0</v>
@@ -3472,7 +3472,7 @@
         <v>0</v>
       </c>
       <c r="H9" t="n">
-        <v>32</v>
+        <v>120</v>
       </c>
       <c r="I9" t="n">
         <v>0</v>
@@ -21184,7 +21184,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -21193,7 +21193,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0</v>
@@ -21246,7 +21246,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -21302,7 +21302,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
@@ -21373,10 +21373,10 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J5" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K5" t="n">
         <v>0</v>
@@ -21432,7 +21432,7 @@
         <v>0</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>0</v>
@@ -21447,7 +21447,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N6" s="3" t="n">
         <v>6</v>
@@ -21488,7 +21488,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -21556,7 +21556,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>33</v>
+        <v>122</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -21571,7 +21571,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -21732,7 +21732,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -21741,7 +21741,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0</v>
@@ -21794,7 +21794,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -21850,7 +21850,7 @@
         </is>
       </c>
       <c r="F4" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>0</v>
@@ -21859,10 +21859,10 @@
         <v>0</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J4" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K4" s="3" t="n">
         <v>0</v>
@@ -21918,7 +21918,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -21933,7 +21933,7 @@
         <v>0</v>
       </c>
       <c r="M5" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="N5" t="n">
         <v>6</v>
@@ -21974,7 +21974,7 @@
         </is>
       </c>
       <c r="F6" s="3" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>0</v>
@@ -22036,7 +22036,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>5</v>
+        <v>11</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -22104,7 +22104,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>33</v>
+        <v>122</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -22119,7 +22119,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -22280,7 +22280,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -22289,7 +22289,7 @@
         <v>0</v>
       </c>
       <c r="K2" s="3" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="L2" s="3" t="n">
         <v>0</v>
@@ -22342,7 +22342,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -22404,7 +22404,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -22419,7 +22419,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="N4" s="3" t="n">
         <v>6</v>
@@ -22460,7 +22460,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G5" t="n">
         <v>0</v>
@@ -22531,10 +22531,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -22584,7 +22584,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -22652,7 +22652,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>33</v>
+        <v>122</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -22667,7 +22667,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>12</v>
@@ -22828,7 +22828,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>11</v>
+        <v>31</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -22890,7 +22890,7 @@
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>2</v>
+        <v>61</v>
       </c>
       <c r="I3" t="n">
         <v>0</v>
@@ -22952,7 +22952,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>22</v>
+        <v>80</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -23017,7 +23017,7 @@
         <v>0</v>
       </c>
       <c r="I5" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -23079,10 +23079,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -23141,7 +23141,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="n">
-        <v>3</v>
+        <v>11</v>
       </c>
       <c r="J7" t="n">
         <v>0</v>
@@ -23200,7 +23200,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>33</v>
+        <v>120</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -23376,7 +23376,7 @@
         <v>0</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>22</v>
+        <v>81</v>
       </c>
       <c r="I2" s="3" t="n">
         <v>0</v>
@@ -23391,7 +23391,7 @@
         <v>0</v>
       </c>
       <c r="M2" s="3" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="N2" s="3" t="n">
         <v>10</v>
@@ -23432,7 +23432,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
@@ -23500,7 +23500,7 @@
         <v>0</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>3</v>
+        <v>61</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>0</v>
@@ -23562,7 +23562,7 @@
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="I5" t="n">
         <v>0</v>
@@ -23571,7 +23571,7 @@
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="L5" t="n">
         <v>0</v>
@@ -23627,10 +23627,10 @@
         <v>0</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="J6" s="3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="K6" s="3" t="n">
         <v>0</v>
@@ -23680,7 +23680,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>3</v>
+        <v>9</v>
       </c>
       <c r="G7" t="n">
         <v>0</v>
@@ -23748,7 +23748,7 @@
         <v>0</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>33</v>
+        <v>122</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>0</v>
@@ -23763,7 +23763,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="3" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="N8" s="3" t="n">
         <v>20</v>

</xml_diff>